<commit_message>
Despliegue de Dashnoard PT2
</commit_message>
<xml_diff>
--- a/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
+++ b/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Reforma_Curricular/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Escritorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12883" documentId="8_{3BAA4E05-85DC-4689-9347-38426449B74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7264511E-D687-423D-BDD4-B3022074C40D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{112CFA50-3194-417D-B4BC-6D8321F8E0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{5D2AA78B-CF8F-4F04-8CED-873384612ABA}"/>
   </bookViews>
@@ -497,7 +497,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4044" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4068" uniqueCount="410">
   <si>
     <t>RC</t>
   </si>
@@ -2926,7 +2926,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="352">
+  <cellXfs count="353">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3709,6 +3709,72 @@
     <xf numFmtId="0" fontId="0" fillId="49" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="68" fillId="26" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -3727,85 +3793,22 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -9107,11 +9110,11 @@
         <v>6</v>
       </c>
       <c r="D3" s="284"/>
-      <c r="E3" s="316" t="s">
+      <c r="E3" s="338" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="317"/>
-      <c r="G3" s="318"/>
+      <c r="F3" s="339"/>
+      <c r="G3" s="340"/>
       <c r="H3" s="282" t="s">
         <v>8</v>
       </c>
@@ -11863,19 +11866,19 @@
       </c>
       <c r="E11" s="141">
         <f>COUNTIFS(Maestro!AQ11:AQ70,"&gt;0",Maestro!AQ11:AQ70,"&lt;1")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" s="142">
         <f t="shared" si="1"/>
-        <v>3.3333333333333333E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="G11" s="143">
         <f>COUNTIF(Maestro!AQ11:AQ70,0)</f>
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H11" s="144">
         <f t="shared" si="2"/>
-        <v>0.96666666666666667</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="I11" s="145">
         <f t="shared" si="3"/>
@@ -12154,21 +12157,21 @@
       <c r="C20" s="121" t="s">
         <v>147</v>
       </c>
-      <c r="D20" s="319" t="s">
+      <c r="D20" s="341" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="319"/>
-      <c r="F20" s="319"/>
-      <c r="G20" s="320" t="s">
+      <c r="E20" s="341"/>
+      <c r="F20" s="341"/>
+      <c r="G20" s="342" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="320"/>
-      <c r="I20" s="320"/>
-      <c r="J20" s="321" t="s">
+      <c r="H20" s="342"/>
+      <c r="I20" s="342"/>
+      <c r="J20" s="343" t="s">
         <v>6</v>
       </c>
-      <c r="K20" s="321"/>
-      <c r="L20" s="321"/>
+      <c r="K20" s="343"/>
+      <c r="L20" s="343"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C21" s="146"/>
@@ -12336,11 +12339,11 @@
       </c>
       <c r="E25" s="154">
         <f>COUNTIFS(Maestro!F11:F70,"Presencial",Maestro!AQ11:AQ70,"&gt;0",Maestro!AQ11:AQ70,"&lt;1")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="155">
         <f>COUNTIFS(Maestro!F11:F70,"Presencial",Maestro!AQ11:AQ70,0)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G25" s="153">
         <f>COUNTIFS(Maestro!F11:F70,"Virtual",Maestro!AQ11:AQ70,"&gt;=1")</f>
@@ -12348,11 +12351,11 @@
       </c>
       <c r="H25" s="154">
         <f>COUNTIFS(Maestro!F11:F70,"Virtual",Maestro!AQ11:AQ70,"&gt;0",Maestro!AQ11:AQ70,"&lt;1")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I25" s="155">
         <f>COUNTIFS(Maestro!F11:F70,"Virtual",Maestro!AQ11:AQ70,0)</f>
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J25" s="153">
         <f>COUNTIFS(Maestro!F11:F70,"Híbrido",Maestro!AQ11:AQ70,"&gt;=1")</f>
@@ -13587,7 +13590,7 @@
       </c>
       <c r="H55" s="157" t="str">
         <f>IF(B55="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B55,Maestro!$I$11:$I$70,Maestro!$AQ$11:$AQ$70,"—"),IF(ISNUMBER(_xlpm.v),TEXT(_xlpm.v,"0%"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v))))))</f>
-        <v>0%</v>
+        <v>10%</v>
       </c>
       <c r="I55" s="157" t="str">
         <f>IF(B55="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B55,Maestro!$I$11:$I$70,Maestro!$AR$11:$AR$70,"—"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v)))))</f>
@@ -14231,7 +14234,7 @@
       </c>
       <c r="H69" s="157" t="str">
         <f>IF(B69="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B69,Maestro!$I$11:$I$70,Maestro!$AQ$11:$AQ$70,"—"),IF(ISNUMBER(_xlpm.v),TEXT(_xlpm.v,"0%"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v))))))</f>
-        <v>0%</v>
+        <v>10%</v>
       </c>
       <c r="I69" s="157" t="str">
         <f>IF(B69="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B69,Maestro!$I$11:$I$70,Maestro!$AR$11:$AR$70,"—"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v)))))</f>
@@ -14277,7 +14280,7 @@
       </c>
       <c r="H70" s="137" t="str">
         <f>IF(B70="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B70,Maestro!$I$11:$I$70,Maestro!$AQ$11:$AQ$70,"—"),IF(ISNUMBER(_xlpm.v),TEXT(_xlpm.v,"0%"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v))))))</f>
-        <v>0%</v>
+        <v>10%</v>
       </c>
       <c r="I70" s="137" t="str">
         <f>IF(B70="","",_xlfn.LET(_xlpm.v,_xlfn.XLOOKUP(B70,Maestro!$I$11:$I$70,Maestro!$AR$11:$AR$70,"—"),IF(_xlpm.v="","—",IF(LEN(_xlpm.v)&gt;1,UPPER(LEFT(_xlpm.v,1))&amp;MID(_xlpm.v,2,LEN(_xlpm.v)),UPPER(_xlpm.v)))))</f>
@@ -15611,43 +15614,43 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:78" ht="32.700000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="335" t="s">
+      <c r="O3" s="333" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="335"/>
-      <c r="Q3" s="335"/>
-      <c r="R3" s="335"/>
-      <c r="S3" s="335"/>
-      <c r="T3" s="335"/>
-      <c r="U3" s="335"/>
-      <c r="V3" s="335"/>
-      <c r="W3" s="335"/>
-      <c r="X3" s="335"/>
-      <c r="Y3" s="335"/>
-      <c r="Z3" s="335"/>
-      <c r="AA3" s="335"/>
-      <c r="AB3" s="335"/>
-      <c r="AC3" s="335"/>
+      <c r="P3" s="333"/>
+      <c r="Q3" s="333"/>
+      <c r="R3" s="333"/>
+      <c r="S3" s="333"/>
+      <c r="T3" s="333"/>
+      <c r="U3" s="333"/>
+      <c r="V3" s="333"/>
+      <c r="W3" s="333"/>
+      <c r="X3" s="333"/>
+      <c r="Y3" s="333"/>
+      <c r="Z3" s="333"/>
+      <c r="AA3" s="333"/>
+      <c r="AB3" s="333"/>
+      <c r="AC3" s="333"/>
     </row>
     <row r="4" spans="3:78" x14ac:dyDescent="0.3">
       <c r="J4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="335"/>
-      <c r="P4" s="335"/>
-      <c r="Q4" s="335"/>
-      <c r="R4" s="335"/>
-      <c r="S4" s="335"/>
-      <c r="T4" s="335"/>
-      <c r="U4" s="335"/>
-      <c r="V4" s="335"/>
-      <c r="W4" s="335"/>
-      <c r="X4" s="335"/>
-      <c r="Y4" s="335"/>
-      <c r="Z4" s="335"/>
-      <c r="AA4" s="335"/>
-      <c r="AB4" s="335"/>
-      <c r="AC4" s="335"/>
+      <c r="O4" s="333"/>
+      <c r="P4" s="333"/>
+      <c r="Q4" s="333"/>
+      <c r="R4" s="333"/>
+      <c r="S4" s="333"/>
+      <c r="T4" s="333"/>
+      <c r="U4" s="333"/>
+      <c r="V4" s="333"/>
+      <c r="W4" s="333"/>
+      <c r="X4" s="333"/>
+      <c r="Y4" s="333"/>
+      <c r="Z4" s="333"/>
+      <c r="AA4" s="333"/>
+      <c r="AB4" s="333"/>
+      <c r="AC4" s="333"/>
     </row>
     <row r="5" spans="3:78" x14ac:dyDescent="0.3">
       <c r="J5" s="3" t="s">
@@ -15676,17 +15679,17 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="331" t="s">
+      <c r="J8" s="324" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="331"/>
-      <c r="L8" s="331"/>
-      <c r="M8" s="331"/>
-      <c r="N8" s="331"/>
-      <c r="O8" s="331"/>
-      <c r="P8" s="331"/>
-      <c r="Q8" s="331"/>
-      <c r="R8" s="331"/>
+      <c r="K8" s="324"/>
+      <c r="L8" s="324"/>
+      <c r="M8" s="324"/>
+      <c r="N8" s="324"/>
+      <c r="O8" s="324"/>
+      <c r="P8" s="324"/>
+      <c r="Q8" s="324"/>
+      <c r="R8" s="324"/>
       <c r="S8" s="5" t="s">
         <v>196</v>
       </c>
@@ -15701,27 +15704,27 @@
       <c r="Z8" s="75"/>
       <c r="AA8" s="75"/>
       <c r="AB8" s="75"/>
-      <c r="AC8" s="336" t="s">
+      <c r="AC8" s="325" t="s">
         <v>198</v>
       </c>
-      <c r="AD8" s="337"/>
-      <c r="AE8" s="337"/>
-      <c r="AF8" s="337"/>
-      <c r="AG8" s="337"/>
-      <c r="AH8" s="338"/>
-      <c r="AI8" s="339" t="s">
+      <c r="AD8" s="326"/>
+      <c r="AE8" s="326"/>
+      <c r="AF8" s="326"/>
+      <c r="AG8" s="326"/>
+      <c r="AH8" s="327"/>
+      <c r="AI8" s="334" t="s">
         <v>199</v>
       </c>
       <c r="AJ8" s="170"/>
       <c r="AK8" s="170"/>
-      <c r="AL8" s="341" t="s">
+      <c r="AL8" s="336" t="s">
         <v>200</v>
       </c>
-      <c r="AM8" s="342"/>
-      <c r="AN8" s="342"/>
-      <c r="AO8" s="342"/>
-      <c r="AP8" s="342"/>
-      <c r="AQ8" s="342"/>
+      <c r="AM8" s="337"/>
+      <c r="AN8" s="337"/>
+      <c r="AO8" s="337"/>
+      <c r="AP8" s="337"/>
+      <c r="AQ8" s="337"/>
       <c r="AR8" s="328" t="s">
         <v>201</v>
       </c>
@@ -15736,89 +15739,89 @@
       <c r="BA8" s="174"/>
       <c r="BB8" s="174"/>
       <c r="BC8" s="174"/>
-      <c r="BD8" s="324" t="s">
+      <c r="BD8" s="321" t="s">
         <v>202</v>
       </c>
-      <c r="BE8" s="324"/>
-      <c r="BF8" s="324"/>
-      <c r="BG8" s="324"/>
-      <c r="BH8" s="324"/>
-      <c r="BI8" s="324"/>
-      <c r="BJ8" s="324"/>
-      <c r="BK8" s="324"/>
-      <c r="BL8" s="324"/>
-      <c r="BM8" s="324"/>
-      <c r="BN8" s="324"/>
-      <c r="BO8" s="324"/>
-      <c r="BP8" s="324"/>
-      <c r="BQ8" s="325" t="s">
+      <c r="BE8" s="321"/>
+      <c r="BF8" s="321"/>
+      <c r="BG8" s="321"/>
+      <c r="BH8" s="321"/>
+      <c r="BI8" s="321"/>
+      <c r="BJ8" s="321"/>
+      <c r="BK8" s="321"/>
+      <c r="BL8" s="321"/>
+      <c r="BM8" s="321"/>
+      <c r="BN8" s="321"/>
+      <c r="BO8" s="321"/>
+      <c r="BP8" s="321"/>
+      <c r="BQ8" s="322" t="s">
         <v>203</v>
       </c>
-      <c r="BR8" s="325"/>
-      <c r="BS8" s="325"/>
+      <c r="BR8" s="322"/>
+      <c r="BS8" s="322"/>
       <c r="BT8" s="14"/>
       <c r="BU8" s="14"/>
       <c r="BV8" s="14"/>
       <c r="BW8" s="14"/>
     </row>
     <row r="9" spans="3:78" s="2" customFormat="1" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="330" t="s">
+      <c r="C9" s="323" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="330"/>
-      <c r="E9" s="330"/>
-      <c r="F9" s="330"/>
-      <c r="G9" s="330"/>
-      <c r="H9" s="330"/>
-      <c r="I9" s="330"/>
-      <c r="J9" s="331" t="s">
+      <c r="D9" s="323"/>
+      <c r="E9" s="323"/>
+      <c r="F9" s="323"/>
+      <c r="G9" s="323"/>
+      <c r="H9" s="323"/>
+      <c r="I9" s="323"/>
+      <c r="J9" s="324" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="331"/>
-      <c r="L9" s="331"/>
-      <c r="M9" s="331"/>
-      <c r="N9" s="331"/>
-      <c r="O9" s="331"/>
-      <c r="P9" s="331"/>
-      <c r="Q9" s="331"/>
-      <c r="R9" s="331"/>
-      <c r="S9" s="332" t="s">
+      <c r="K9" s="324"/>
+      <c r="L9" s="324"/>
+      <c r="M9" s="324"/>
+      <c r="N9" s="324"/>
+      <c r="O9" s="324"/>
+      <c r="P9" s="324"/>
+      <c r="Q9" s="324"/>
+      <c r="R9" s="324"/>
+      <c r="S9" s="347" t="s">
         <v>205</v>
       </c>
-      <c r="T9" s="333" t="s">
+      <c r="T9" s="344" t="s">
         <v>206</v>
       </c>
-      <c r="U9" s="333" t="s">
+      <c r="U9" s="344" t="s">
         <v>158</v>
       </c>
-      <c r="V9" s="333" t="s">
+      <c r="V9" s="344" t="s">
         <v>207</v>
       </c>
       <c r="W9" s="199"/>
       <c r="X9" s="199"/>
       <c r="Y9" s="199"/>
       <c r="Z9" s="199"/>
-      <c r="AA9" s="336" t="s">
+      <c r="AA9" s="325" t="s">
         <v>208</v>
       </c>
-      <c r="AB9" s="337"/>
-      <c r="AC9" s="337"/>
-      <c r="AD9" s="337"/>
-      <c r="AE9" s="337"/>
-      <c r="AF9" s="337"/>
-      <c r="AG9" s="337"/>
-      <c r="AH9" s="338"/>
-      <c r="AI9" s="340"/>
+      <c r="AB9" s="326"/>
+      <c r="AC9" s="326"/>
+      <c r="AD9" s="326"/>
+      <c r="AE9" s="326"/>
+      <c r="AF9" s="326"/>
+      <c r="AG9" s="326"/>
+      <c r="AH9" s="327"/>
+      <c r="AI9" s="335"/>
       <c r="AJ9" s="172"/>
       <c r="AK9" s="172"/>
-      <c r="AL9" s="343" t="s">
+      <c r="AL9" s="346" t="s">
         <v>209</v>
       </c>
-      <c r="AM9" s="343"/>
-      <c r="AN9" s="343"/>
-      <c r="AO9" s="343"/>
-      <c r="AP9" s="343"/>
-      <c r="AQ9" s="343"/>
+      <c r="AM9" s="346"/>
+      <c r="AN9" s="346"/>
+      <c r="AO9" s="346"/>
+      <c r="AP9" s="346"/>
+      <c r="AQ9" s="346"/>
       <c r="AR9" s="329" t="s">
         <v>201</v>
       </c>
@@ -15833,36 +15836,36 @@
       <c r="BA9" s="175"/>
       <c r="BB9" s="175"/>
       <c r="BC9" s="175"/>
-      <c r="BD9" s="326" t="s">
+      <c r="BD9" s="317" t="s">
         <v>210</v>
       </c>
-      <c r="BE9" s="326"/>
-      <c r="BF9" s="326"/>
-      <c r="BG9" s="326"/>
-      <c r="BH9" s="326"/>
-      <c r="BI9" s="326"/>
-      <c r="BJ9" s="326"/>
-      <c r="BK9" s="326"/>
-      <c r="BL9" s="326"/>
-      <c r="BM9" s="326"/>
-      <c r="BN9" s="326"/>
-      <c r="BO9" s="326"/>
-      <c r="BP9" s="326"/>
-      <c r="BQ9" s="327" t="s">
+      <c r="BE9" s="317"/>
+      <c r="BF9" s="317"/>
+      <c r="BG9" s="317"/>
+      <c r="BH9" s="317"/>
+      <c r="BI9" s="317"/>
+      <c r="BJ9" s="317"/>
+      <c r="BK9" s="317"/>
+      <c r="BL9" s="317"/>
+      <c r="BM9" s="317"/>
+      <c r="BN9" s="317"/>
+      <c r="BO9" s="317"/>
+      <c r="BP9" s="317"/>
+      <c r="BQ9" s="320" t="s">
         <v>211</v>
       </c>
-      <c r="BR9" s="327"/>
-      <c r="BS9" s="327"/>
-      <c r="BT9" s="322" t="s">
+      <c r="BR9" s="320"/>
+      <c r="BS9" s="320"/>
+      <c r="BT9" s="348" t="s">
         <v>212</v>
       </c>
-      <c r="BU9" s="322" t="s">
+      <c r="BU9" s="348" t="s">
         <v>213</v>
       </c>
-      <c r="BV9" s="322" t="s">
+      <c r="BV9" s="348" t="s">
         <v>214</v>
       </c>
-      <c r="BW9" s="323" t="s">
+      <c r="BW9" s="349" t="s">
         <v>215</v>
       </c>
       <c r="BZ9" s="2" t="s">
@@ -15918,10 +15921,10 @@
       <c r="R10" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="S10" s="332"/>
-      <c r="T10" s="334"/>
-      <c r="U10" s="334"/>
-      <c r="V10" s="334"/>
+      <c r="S10" s="347"/>
+      <c r="T10" s="345"/>
+      <c r="U10" s="345"/>
+      <c r="V10" s="345"/>
       <c r="W10" s="173" t="s">
         <v>205</v>
       </c>
@@ -16047,10 +16050,10 @@
       <c r="BS10" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="BT10" s="322"/>
-      <c r="BU10" s="322"/>
-      <c r="BV10" s="322"/>
-      <c r="BW10" s="323"/>
+      <c r="BT10" s="348"/>
+      <c r="BU10" s="348"/>
+      <c r="BV10" s="348"/>
+      <c r="BW10" s="349"/>
     </row>
     <row r="11" spans="3:78" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C11" s="22" t="str">
@@ -16455,7 +16458,7 @@
       </c>
       <c r="AG12" s="12" t="str" cm="1">
         <f t="array" ref="AG12">IFERROR(_xlfn.XLOOKUP($I12,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AG$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>No aplica</v>
+        <v>No</v>
       </c>
       <c r="AH12" s="12" t="str" cm="1">
         <f t="array" ref="AH12">IFERROR(_xlfn.XLOOKUP($I12,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AH$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -16739,7 +16742,7 @@
       </c>
       <c r="AG13" s="12" t="str" cm="1">
         <f t="array" ref="AG13">IFERROR(_xlfn.XLOOKUP($I13,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AG$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Si</v>
+        <v>Sí</v>
       </c>
       <c r="AH13" s="12" t="str" cm="1">
         <f t="array" ref="AH13">IFERROR(_xlfn.XLOOKUP($I13,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AH$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -16849,7 +16852,7 @@
       </c>
       <c r="BJ13" s="12" t="str" cm="1">
         <f t="array" ref="BJ13">IFERROR(_xlfn.XLOOKUP($I13,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK13" s="12" cm="1">
         <f t="array" ref="BK13">IFERROR(_xlfn.XLOOKUP($I13,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -17133,7 +17136,7 @@
       </c>
       <c r="BJ14" s="12" t="str" cm="1">
         <f t="array" ref="BJ14">IFERROR(_xlfn.XLOOKUP($I14,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK14" s="12" cm="1">
         <f t="array" ref="BK14">IFERROR(_xlfn.XLOOKUP($I14,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -19690,7 +19693,7 @@
       </c>
       <c r="BJ23" s="12" t="str" cm="1">
         <f t="array" ref="BJ23">IFERROR(_xlfn.XLOOKUP($I23,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK23" s="12" cm="1">
         <f t="array" ref="BK23">IFERROR(_xlfn.XLOOKUP($I23,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -20258,7 +20261,7 @@
       </c>
       <c r="BJ25" s="12" t="str" cm="1">
         <f t="array" ref="BJ25">IFERROR(_xlfn.XLOOKUP($I25,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK25" s="12" cm="1">
         <f t="array" ref="BK25">IFERROR(_xlfn.XLOOKUP($I25,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -21614,15 +21617,15 @@
       </c>
       <c r="AT30" s="12" t="str" cm="1">
         <f t="array" ref="AT30">IFERROR(_xlfn.XLOOKUP($I30,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AT$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AU30" s="12" t="str" cm="1">
         <f t="array" ref="AU30">IFERROR(_xlfn.XLOOKUP($I30,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AU$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AV30" s="12" t="str" cm="1">
         <f t="array" ref="AV30">IFERROR(_xlfn.XLOOKUP($I30,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AV$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AW30" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I30,Borrador!$I$11:$I$70,Borrador!$AQ$11:$AQ$70,""),"")</f>
@@ -21887,7 +21890,7 @@
       </c>
       <c r="AQ31" s="11" cm="1">
         <f t="array" ref="AQ31">IFERROR(_xlfn.XLOOKUP($I31,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AQ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AR31" s="12" t="str" cm="1">
         <f t="array" ref="AR31">IFERROR(_xlfn.XLOOKUP($I31,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AR$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -21919,11 +21922,11 @@
       </c>
       <c r="AY31" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I31,Borrador!$I$11:$I$70,Borrador!$AS$11:$AS$70,""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AZ31" s="11" cm="1">
         <f t="array" ref="AZ31">IFERROR(_xlfn.XLOOKUP($I31,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AZ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BA31" s="11" cm="1">
         <f t="array" ref="BA31">IFERROR(_xlfn.XLOOKUP($I31,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BA$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -23388,7 +23391,7 @@
       </c>
       <c r="BJ36" s="12" t="str" cm="1">
         <f t="array" ref="BJ36">IFERROR(_xlfn.XLOOKUP($I36,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK36" s="12" cm="1">
         <f t="array" ref="BK36">IFERROR(_xlfn.XLOOKUP($I36,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -25874,7 +25877,7 @@
       </c>
       <c r="AQ45" s="11" cm="1">
         <f t="array" ref="AQ45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AQ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AR45" s="12" t="str" cm="1">
         <f t="array" ref="AR45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AR$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -25886,15 +25889,15 @@
       </c>
       <c r="AT45" s="12" t="str" cm="1">
         <f t="array" ref="AT45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AT$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AU45" s="12" t="str" cm="1">
         <f t="array" ref="AU45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AU$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AV45" s="12" t="str" cm="1">
         <f t="array" ref="AV45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AV$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AW45" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,Borrador!$AQ$11:$AQ$70,""),"")</f>
@@ -25906,11 +25909,11 @@
       </c>
       <c r="AY45" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,Borrador!$AS$11:$AS$70,""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AZ45" s="11" cm="1">
         <f t="array" ref="AZ45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AZ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BA45" s="11" t="str" cm="1">
         <f t="array" ref="BA45">IFERROR(_xlfn.XLOOKUP($I45,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BA$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -26158,7 +26161,7 @@
       </c>
       <c r="AQ46" s="11" cm="1">
         <f t="array" ref="AQ46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AQ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AR46" s="12" t="str" cm="1">
         <f t="array" ref="AR46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AR$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -26170,15 +26173,15 @@
       </c>
       <c r="AT46" s="12" t="str" cm="1">
         <f t="array" ref="AT46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AT$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AU46" s="12" t="str" cm="1">
         <f t="array" ref="AU46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AU$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AV46" s="12" t="str" cm="1">
         <f t="array" ref="AV46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AV$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>sin iniciar</v>
+        <v>en proceso</v>
       </c>
       <c r="AW46" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,Borrador!$AQ$11:$AQ$70,""),"")</f>
@@ -26190,11 +26193,11 @@
       </c>
       <c r="AY46" s="12">
         <f>IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,Borrador!$AS$11:$AS$70,""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AZ46" s="11" cm="1">
         <f t="array" ref="AZ46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AZ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BA46" s="11" cm="1">
         <f t="array" ref="BA46">IFERROR(_xlfn.XLOOKUP($I46,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BA$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -28222,7 +28225,7 @@
       </c>
       <c r="BJ53" s="12" t="str" cm="1">
         <f t="array" ref="BJ53">IFERROR(_xlfn.XLOOKUP($I53,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>No aplica</v>
       </c>
       <c r="BK53" s="12" cm="1">
         <f t="array" ref="BK53">IFERROR(_xlfn.XLOOKUP($I53,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -28680,7 +28683,7 @@
       </c>
       <c r="AG55" s="12" t="str" cm="1">
         <f t="array" ref="AG55">IFERROR(_xlfn.XLOOKUP($I55,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AG$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>No aplica</v>
+        <v>No</v>
       </c>
       <c r="AH55" s="12" t="str" cm="1">
         <f t="array" ref="AH55">IFERROR(_xlfn.XLOOKUP($I55,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AH$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -28788,9 +28791,9 @@
         <f t="array" ref="BI55">IFERROR(_xlfn.XLOOKUP($I55,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BI$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
         <v>sin iniciar</v>
       </c>
-      <c r="BJ55" s="12" t="str" cm="1">
+      <c r="BJ55" s="12" cm="1">
         <f t="array" ref="BJ55">IFERROR(_xlfn.XLOOKUP($I55,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BJ$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>Validar datos de Aulas Master</v>
+        <v>1</v>
       </c>
       <c r="BK55" s="12" cm="1">
         <f t="array" ref="BK55">IFERROR(_xlfn.XLOOKUP($I55,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(BK$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -31236,7 +31239,7 @@
       </c>
       <c r="AG64" s="12" t="str" cm="1">
         <f t="array" ref="AG64">IFERROR(_xlfn.XLOOKUP($I64,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AG$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
-        <v>No aplica</v>
+        <v>No</v>
       </c>
       <c r="AH64" s="12" t="str" cm="1">
         <f t="array" ref="AH64">IFERROR(_xlfn.XLOOKUP($I64,Borrador!$I$11:$I$70,_xlfn.XLOOKUP(AH$10,Borrador!$C$10:$BL$10,Borrador!$C$11:$BL$70,"",0,1),""),"")</f>
@@ -33090,6 +33093,21 @@
   </sheetData>
   <autoFilter ref="C10:BZ10" xr:uid="{0DE7F4C8-C4D9-4718-9A45-DE15ED66A68A}"/>
   <mergeCells count="23">
+    <mergeCell ref="BU9:BU10"/>
+    <mergeCell ref="BV9:BV10"/>
+    <mergeCell ref="BW9:BW10"/>
+    <mergeCell ref="BD8:BP8"/>
+    <mergeCell ref="BQ8:BS8"/>
+    <mergeCell ref="BD9:BP9"/>
+    <mergeCell ref="BQ9:BS9"/>
+    <mergeCell ref="BT9:BT10"/>
+    <mergeCell ref="AR8:AZ8"/>
+    <mergeCell ref="AR9:AZ9"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:R9"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
     <mergeCell ref="O3:AC4"/>
     <mergeCell ref="J8:R8"/>
     <mergeCell ref="AC8:AH8"/>
@@ -33098,21 +33116,6 @@
     <mergeCell ref="V9:V10"/>
     <mergeCell ref="AA9:AH9"/>
     <mergeCell ref="AL9:AQ9"/>
-    <mergeCell ref="AR8:AZ8"/>
-    <mergeCell ref="AR9:AZ9"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:R9"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="BU9:BU10"/>
-    <mergeCell ref="BV9:BV10"/>
-    <mergeCell ref="BW9:BW10"/>
-    <mergeCell ref="BD8:BP8"/>
-    <mergeCell ref="BQ8:BS8"/>
-    <mergeCell ref="BD9:BP9"/>
-    <mergeCell ref="BQ9:BS9"/>
-    <mergeCell ref="BT9:BT10"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M69 M70:N70">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="En Proceso">
@@ -33232,33 +33235,33 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:65" ht="32.700000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="335" t="s">
+      <c r="O3" s="333" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="335"/>
-      <c r="Q3" s="335"/>
-      <c r="R3" s="335"/>
-      <c r="S3" s="335"/>
-      <c r="T3" s="335"/>
-      <c r="U3" s="335"/>
-      <c r="V3" s="335"/>
-      <c r="W3" s="335"/>
-      <c r="X3" s="335"/>
+      <c r="P3" s="333"/>
+      <c r="Q3" s="333"/>
+      <c r="R3" s="333"/>
+      <c r="S3" s="333"/>
+      <c r="T3" s="333"/>
+      <c r="U3" s="333"/>
+      <c r="V3" s="333"/>
+      <c r="W3" s="333"/>
+      <c r="X3" s="333"/>
     </row>
     <row r="4" spans="3:65" ht="14.4" x14ac:dyDescent="0.3">
       <c r="J4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="335"/>
-      <c r="P4" s="335"/>
-      <c r="Q4" s="335"/>
-      <c r="R4" s="335"/>
-      <c r="S4" s="335"/>
-      <c r="T4" s="335"/>
-      <c r="U4" s="335"/>
-      <c r="V4" s="335"/>
-      <c r="W4" s="335"/>
-      <c r="X4" s="335"/>
+      <c r="O4" s="333"/>
+      <c r="P4" s="333"/>
+      <c r="Q4" s="333"/>
+      <c r="R4" s="333"/>
+      <c r="S4" s="333"/>
+      <c r="T4" s="333"/>
+      <c r="U4" s="333"/>
+      <c r="V4" s="333"/>
+      <c r="W4" s="333"/>
+      <c r="X4" s="333"/>
     </row>
     <row r="5" spans="3:65" ht="14.4" x14ac:dyDescent="0.3">
       <c r="J5" s="3" t="s">
@@ -33287,16 +33290,16 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="331" t="s">
+      <c r="J8" s="324" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="331"/>
-      <c r="L8" s="331"/>
-      <c r="M8" s="331"/>
-      <c r="N8" s="331"/>
-      <c r="O8" s="331"/>
-      <c r="P8" s="331"/>
-      <c r="Q8" s="331"/>
+      <c r="K8" s="324"/>
+      <c r="L8" s="324"/>
+      <c r="M8" s="324"/>
+      <c r="N8" s="324"/>
+      <c r="O8" s="324"/>
+      <c r="P8" s="324"/>
+      <c r="Q8" s="324"/>
       <c r="R8" s="5" t="s">
         <v>196</v>
       </c>
@@ -33307,26 +33310,26 @@
       </c>
       <c r="V8" s="75"/>
       <c r="W8" s="75"/>
-      <c r="X8" s="336" t="s">
+      <c r="X8" s="325" t="s">
         <v>198</v>
       </c>
-      <c r="Y8" s="337"/>
-      <c r="Z8" s="337"/>
-      <c r="AA8" s="337"/>
-      <c r="AB8" s="338"/>
-      <c r="AC8" s="339" t="s">
+      <c r="Y8" s="326"/>
+      <c r="Z8" s="326"/>
+      <c r="AA8" s="326"/>
+      <c r="AB8" s="327"/>
+      <c r="AC8" s="334" t="s">
         <v>199</v>
       </c>
       <c r="AD8" s="170"/>
       <c r="AE8" s="170"/>
-      <c r="AF8" s="341" t="s">
+      <c r="AF8" s="336" t="s">
         <v>200</v>
       </c>
-      <c r="AG8" s="342"/>
-      <c r="AH8" s="342"/>
-      <c r="AI8" s="342"/>
-      <c r="AJ8" s="342"/>
-      <c r="AK8" s="342"/>
+      <c r="AG8" s="337"/>
+      <c r="AH8" s="337"/>
+      <c r="AI8" s="337"/>
+      <c r="AJ8" s="337"/>
+      <c r="AK8" s="337"/>
       <c r="AL8" s="328" t="s">
         <v>201</v>
       </c>
@@ -33337,74 +33340,74 @@
       <c r="AQ8" s="328"/>
       <c r="AR8" s="328"/>
       <c r="AS8" s="328"/>
-      <c r="AT8" s="324" t="s">
+      <c r="AT8" s="321" t="s">
         <v>202</v>
       </c>
-      <c r="AU8" s="324"/>
-      <c r="AV8" s="324"/>
-      <c r="AW8" s="324"/>
-      <c r="AX8" s="324"/>
-      <c r="AY8" s="324"/>
-      <c r="AZ8" s="324"/>
-      <c r="BA8" s="324"/>
-      <c r="BB8" s="324"/>
-      <c r="BC8" s="325" t="s">
+      <c r="AU8" s="321"/>
+      <c r="AV8" s="321"/>
+      <c r="AW8" s="321"/>
+      <c r="AX8" s="321"/>
+      <c r="AY8" s="321"/>
+      <c r="AZ8" s="321"/>
+      <c r="BA8" s="321"/>
+      <c r="BB8" s="321"/>
+      <c r="BC8" s="322" t="s">
         <v>203</v>
       </c>
-      <c r="BD8" s="325"/>
-      <c r="BE8" s="325"/>
-      <c r="BF8" s="325"/>
-      <c r="BG8" s="325"/>
-      <c r="BH8" s="325"/>
+      <c r="BD8" s="322"/>
+      <c r="BE8" s="322"/>
+      <c r="BF8" s="322"/>
+      <c r="BG8" s="322"/>
+      <c r="BH8" s="322"/>
       <c r="BI8" s="14"/>
       <c r="BJ8" s="14"/>
       <c r="BK8" s="14"/>
       <c r="BL8" s="14"/>
     </row>
     <row r="9" spans="3:65" s="2" customFormat="1" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="330" t="s">
+      <c r="C9" s="323" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="330"/>
-      <c r="E9" s="330"/>
-      <c r="F9" s="330"/>
-      <c r="G9" s="330"/>
-      <c r="H9" s="330"/>
-      <c r="I9" s="330"/>
-      <c r="J9" s="331" t="s">
+      <c r="D9" s="323"/>
+      <c r="E9" s="323"/>
+      <c r="F9" s="323"/>
+      <c r="G9" s="323"/>
+      <c r="H9" s="323"/>
+      <c r="I9" s="323"/>
+      <c r="J9" s="324" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="331"/>
-      <c r="L9" s="331"/>
-      <c r="M9" s="331"/>
-      <c r="N9" s="331"/>
-      <c r="O9" s="331"/>
-      <c r="P9" s="331"/>
-      <c r="Q9" s="331"/>
+      <c r="K9" s="324"/>
+      <c r="L9" s="324"/>
+      <c r="M9" s="324"/>
+      <c r="N9" s="324"/>
+      <c r="O9" s="324"/>
+      <c r="P9" s="324"/>
+      <c r="Q9" s="324"/>
       <c r="R9" s="81"/>
       <c r="S9" s="82"/>
       <c r="T9" s="82"/>
       <c r="U9" s="82"/>
-      <c r="V9" s="336" t="s">
+      <c r="V9" s="325" t="s">
         <v>208</v>
       </c>
-      <c r="W9" s="337"/>
-      <c r="X9" s="337"/>
-      <c r="Y9" s="337"/>
-      <c r="Z9" s="337"/>
-      <c r="AA9" s="337"/>
-      <c r="AB9" s="338"/>
-      <c r="AC9" s="340"/>
-      <c r="AD9" s="346" t="s">
+      <c r="W9" s="326"/>
+      <c r="X9" s="326"/>
+      <c r="Y9" s="326"/>
+      <c r="Z9" s="326"/>
+      <c r="AA9" s="326"/>
+      <c r="AB9" s="327"/>
+      <c r="AC9" s="335"/>
+      <c r="AD9" s="330" t="s">
         <v>209</v>
       </c>
-      <c r="AE9" s="347"/>
-      <c r="AF9" s="347"/>
-      <c r="AG9" s="347"/>
-      <c r="AH9" s="347"/>
-      <c r="AI9" s="347"/>
-      <c r="AJ9" s="347"/>
-      <c r="AK9" s="348"/>
+      <c r="AE9" s="331"/>
+      <c r="AF9" s="331"/>
+      <c r="AG9" s="331"/>
+      <c r="AH9" s="331"/>
+      <c r="AI9" s="331"/>
+      <c r="AJ9" s="331"/>
+      <c r="AK9" s="332"/>
       <c r="AL9" s="329" t="s">
         <v>201</v>
       </c>
@@ -33415,25 +33418,25 @@
       <c r="AQ9" s="329"/>
       <c r="AR9" s="329"/>
       <c r="AS9" s="329"/>
-      <c r="AT9" s="326" t="s">
+      <c r="AT9" s="317" t="s">
         <v>210</v>
       </c>
-      <c r="AU9" s="326"/>
-      <c r="AV9" s="326"/>
-      <c r="AW9" s="326"/>
-      <c r="AX9" s="326"/>
-      <c r="AY9" s="344"/>
-      <c r="AZ9" s="344"/>
-      <c r="BA9" s="344"/>
-      <c r="BB9" s="344"/>
-      <c r="BC9" s="345" t="s">
+      <c r="AU9" s="317"/>
+      <c r="AV9" s="317"/>
+      <c r="AW9" s="317"/>
+      <c r="AX9" s="317"/>
+      <c r="AY9" s="318"/>
+      <c r="AZ9" s="318"/>
+      <c r="BA9" s="318"/>
+      <c r="BB9" s="318"/>
+      <c r="BC9" s="319" t="s">
         <v>211</v>
       </c>
-      <c r="BD9" s="327"/>
-      <c r="BE9" s="327"/>
-      <c r="BF9" s="327"/>
-      <c r="BG9" s="327"/>
-      <c r="BH9" s="327"/>
+      <c r="BD9" s="320"/>
+      <c r="BE9" s="320"/>
+      <c r="BF9" s="320"/>
+      <c r="BG9" s="320"/>
+      <c r="BH9" s="320"/>
       <c r="BI9" s="83" t="s">
         <v>212</v>
       </c>
@@ -34006,7 +34009,7 @@
         <v>312</v>
       </c>
       <c r="AA13" s="190" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="AB13" s="190" t="s">
         <v>312</v>
@@ -34158,7 +34161,7 @@
         <v>317</v>
       </c>
       <c r="AA14" s="190" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="AB14" s="190" t="s">
         <v>318</v>
@@ -34217,9 +34220,8 @@
       </c>
       <c r="AZ14" s="12"/>
       <c r="BA14" s="12"/>
-      <c r="BB14" s="185" t="str">
-        <f>IFERROR(AW14/AV14,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB14" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC14" s="12"/>
       <c r="BD14" s="177"/>
@@ -34357,9 +34359,8 @@
       </c>
       <c r="AZ15" s="12"/>
       <c r="BA15" s="12"/>
-      <c r="BB15" s="185" t="str">
-        <f>IFERROR(AW15/AV15,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB15" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC15" s="12"/>
       <c r="BD15" s="177"/>
@@ -35618,9 +35619,8 @@
       </c>
       <c r="AZ24" s="12"/>
       <c r="BA24" s="12"/>
-      <c r="BB24" s="185" t="str">
-        <f>IFERROR(AW24/AV24,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB24" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC24" s="12"/>
       <c r="BD24" s="177"/>
@@ -35899,9 +35899,8 @@
       </c>
       <c r="AZ26" s="12"/>
       <c r="BA26" s="12"/>
-      <c r="BB26" s="185" t="str">
-        <f>IFERROR(AW26/AV26,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB26" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC26" s="12"/>
       <c r="BD26" s="177"/>
@@ -36597,13 +36596,13 @@
         <v>194</v>
       </c>
       <c r="AN31" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AO31" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AP31" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AQ31" s="12"/>
       <c r="AR31" s="12"/>
@@ -36765,8 +36764,8 @@
       </c>
       <c r="AQ32" s="12"/>
       <c r="AR32" s="12"/>
-      <c r="AS32" s="11">
-        <v>0</v>
+      <c r="AS32" s="70">
+        <v>0.1</v>
       </c>
       <c r="AT32" s="12" t="s">
         <v>194</v>
@@ -37435,7 +37434,9 @@
       <c r="AC37" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD37" s="12"/>
+      <c r="AD37" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE37" s="12"/>
       <c r="AF37" s="11"/>
       <c r="AG37" s="11"/>
@@ -37484,9 +37485,8 @@
       </c>
       <c r="AZ37" s="12"/>
       <c r="BA37" s="12"/>
-      <c r="BB37" s="185" t="str">
-        <f>IFERROR(AW37/AV37,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB37" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC37" s="12"/>
       <c r="BD37" s="177"/>
@@ -37574,7 +37574,9 @@
       <c r="AC38" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD38" s="12"/>
+      <c r="AD38" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE38" s="12"/>
       <c r="AF38" s="11" t="s">
         <v>312</v>
@@ -38167,7 +38169,9 @@
       <c r="AC42" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD42" s="12"/>
+      <c r="AD42" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE42" s="12"/>
       <c r="AF42" s="11" t="s">
         <v>312</v>
@@ -38607,7 +38611,9 @@
       <c r="AC45" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD45" s="12"/>
+      <c r="AD45" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE45" s="12"/>
       <c r="AF45" s="11" t="s">
         <v>312</v>
@@ -38731,7 +38737,9 @@
       <c r="AC46" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD46" s="12"/>
+      <c r="AD46" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE46" s="12"/>
       <c r="AF46" s="11" t="s">
         <v>312</v>
@@ -38754,18 +38762,18 @@
         <v>194</v>
       </c>
       <c r="AN46" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AO46" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AP46" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AQ46" s="12"/>
       <c r="AR46" s="12"/>
       <c r="AS46" s="70">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AT46" s="12"/>
       <c r="AU46" s="12"/>
@@ -38896,18 +38904,18 @@
         <v>194</v>
       </c>
       <c r="AN47" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AO47" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AP47" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AQ47" s="12"/>
       <c r="AR47" s="12"/>
       <c r="AS47" s="70">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AT47" s="12" t="s">
         <v>194</v>
@@ -39171,7 +39179,9 @@
       <c r="AC49" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD49" s="12"/>
+      <c r="AD49" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE49" s="12"/>
       <c r="AF49" s="11" t="s">
         <v>312</v>
@@ -39295,7 +39305,9 @@
       <c r="AC50" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD50" s="12"/>
+      <c r="AD50" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE50" s="12"/>
       <c r="AF50" s="11" t="s">
         <v>312</v>
@@ -39584,7 +39596,9 @@
       <c r="AC52" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD52" s="12"/>
+      <c r="AD52" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE52" s="12"/>
       <c r="AF52" s="11" t="s">
         <v>312</v>
@@ -39720,7 +39734,9 @@
       <c r="AC53" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD53" s="12"/>
+      <c r="AD53" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE53" s="12"/>
       <c r="AF53" s="11" t="s">
         <v>312</v>
@@ -39897,7 +39913,7 @@
         <v>194</v>
       </c>
       <c r="AV54" s="79">
-        <f t="shared" si="1"/>
+        <f>AH54</f>
         <v>0</v>
       </c>
       <c r="AW54" s="184">
@@ -39911,9 +39927,8 @@
       </c>
       <c r="AZ54" s="12"/>
       <c r="BA54" s="12"/>
-      <c r="BB54" s="185" t="str">
-        <f>IFERROR(AW54/AV54,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB54" s="185" t="s">
+        <v>312</v>
       </c>
       <c r="BC54" s="12"/>
       <c r="BD54" s="177"/>
@@ -40001,7 +40016,9 @@
       <c r="AC55" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD55" s="12"/>
+      <c r="AD55" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE55" s="12"/>
       <c r="AF55" s="11" t="s">
         <v>312</v>
@@ -40119,7 +40136,7 @@
         <v>312</v>
       </c>
       <c r="AA56" s="190" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="AB56" s="190" t="s">
         <v>312</v>
@@ -40178,9 +40195,8 @@
       </c>
       <c r="AZ56" s="12"/>
       <c r="BA56" s="12"/>
-      <c r="BB56" s="185" t="str">
-        <f>IFERROR(AW56/AV56,"Validar datos de Aulas Master")</f>
-        <v>Validar datos de Aulas Master</v>
+      <c r="BB56" s="185">
+        <v>1</v>
       </c>
       <c r="BC56" s="12"/>
       <c r="BD56" s="177"/>
@@ -40419,7 +40435,9 @@
       <c r="AC58" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD58" s="12"/>
+      <c r="AD58" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE58" s="12"/>
       <c r="AF58" s="11" t="s">
         <v>312</v>
@@ -40543,7 +40561,9 @@
       <c r="AC59" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD59" s="12"/>
+      <c r="AD59" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE59" s="12"/>
       <c r="AF59" s="11" t="s">
         <v>312</v>
@@ -40667,7 +40687,9 @@
       <c r="AC60" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD60" s="12"/>
+      <c r="AD60" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE60" s="12"/>
       <c r="AF60" s="11" t="s">
         <v>312</v>
@@ -40791,7 +40813,9 @@
       <c r="AC61" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD61" s="12"/>
+      <c r="AD61" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE61" s="12"/>
       <c r="AF61" s="11" t="s">
         <v>312</v>
@@ -41078,7 +41102,9 @@
       <c r="AC63" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD63" s="12"/>
+      <c r="AD63" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE63" s="12"/>
       <c r="AF63" s="11" t="s">
         <v>312</v>
@@ -41353,7 +41379,7 @@
         <v>312</v>
       </c>
       <c r="AA65" s="190" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="AB65" s="190" t="s">
         <v>312</v>
@@ -41510,7 +41536,9 @@
       <c r="AC66" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD66" s="12"/>
+      <c r="AD66" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE66" s="12"/>
       <c r="AF66" s="11" t="s">
         <v>312</v>
@@ -41634,7 +41662,9 @@
       <c r="AC67" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD67" s="12"/>
+      <c r="AD67" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE67" s="12"/>
       <c r="AF67" s="11" t="s">
         <v>312</v>
@@ -41758,7 +41788,9 @@
       <c r="AC68" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="AD68" s="12"/>
+      <c r="AD68" s="12" t="s">
+        <v>343</v>
+      </c>
       <c r="AE68" s="12"/>
       <c r="AF68" s="11" t="s">
         <v>312</v>
@@ -42118,7 +42150,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="71" spans="3:63" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="3:63" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="BB71" s="316"/>
+    </row>
     <row r="72" spans="3:63" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="73" spans="3:63" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="74" spans="3:63" ht="14.4" x14ac:dyDescent="0.3"/>
@@ -42133,6 +42167,11 @@
     <row r="83" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="O3:X4"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="X8:AB8"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AF8:AK8"/>
     <mergeCell ref="AT9:BB9"/>
     <mergeCell ref="BC9:BH9"/>
     <mergeCell ref="AT8:BB8"/>
@@ -42143,11 +42182,6 @@
     <mergeCell ref="AL8:AS8"/>
     <mergeCell ref="AL9:AS9"/>
     <mergeCell ref="AD9:AK9"/>
-    <mergeCell ref="O3:X4"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="X8:AB8"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AF8:AK8"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M67 M69 M70:N70">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="En Proceso">
@@ -42233,33 +42267,33 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:54" ht="32.700000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="335" t="s">
+      <c r="O3" s="333" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="335"/>
-      <c r="Q3" s="335"/>
-      <c r="R3" s="335"/>
-      <c r="S3" s="335"/>
-      <c r="T3" s="335"/>
-      <c r="U3" s="335"/>
-      <c r="V3" s="335"/>
-      <c r="W3" s="335"/>
-      <c r="X3" s="335"/>
+      <c r="P3" s="333"/>
+      <c r="Q3" s="333"/>
+      <c r="R3" s="333"/>
+      <c r="S3" s="333"/>
+      <c r="T3" s="333"/>
+      <c r="U3" s="333"/>
+      <c r="V3" s="333"/>
+      <c r="W3" s="333"/>
+      <c r="X3" s="333"/>
     </row>
     <row r="4" spans="3:54" x14ac:dyDescent="0.3">
       <c r="J4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="335"/>
-      <c r="P4" s="335"/>
-      <c r="Q4" s="335"/>
-      <c r="R4" s="335"/>
-      <c r="S4" s="335"/>
-      <c r="T4" s="335"/>
-      <c r="U4" s="335"/>
-      <c r="V4" s="335"/>
-      <c r="W4" s="335"/>
-      <c r="X4" s="335"/>
+      <c r="O4" s="333"/>
+      <c r="P4" s="333"/>
+      <c r="Q4" s="333"/>
+      <c r="R4" s="333"/>
+      <c r="S4" s="333"/>
+      <c r="T4" s="333"/>
+      <c r="U4" s="333"/>
+      <c r="V4" s="333"/>
+      <c r="W4" s="333"/>
+      <c r="X4" s="333"/>
     </row>
     <row r="5" spans="3:54" x14ac:dyDescent="0.3">
       <c r="J5" s="3" t="s">
@@ -42288,16 +42322,16 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="331" t="s">
+      <c r="J8" s="324" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="331"/>
-      <c r="L8" s="331"/>
-      <c r="M8" s="331"/>
-      <c r="N8" s="331"/>
-      <c r="O8" s="331"/>
-      <c r="P8" s="331"/>
-      <c r="Q8" s="331"/>
+      <c r="K8" s="324"/>
+      <c r="L8" s="324"/>
+      <c r="M8" s="324"/>
+      <c r="N8" s="324"/>
+      <c r="O8" s="324"/>
+      <c r="P8" s="324"/>
+      <c r="Q8" s="324"/>
       <c r="R8" s="5" t="s">
         <v>196</v>
       </c>
@@ -42308,23 +42342,23 @@
       </c>
       <c r="V8" s="75"/>
       <c r="W8" s="75"/>
-      <c r="X8" s="336" t="s">
+      <c r="X8" s="325" t="s">
         <v>198</v>
       </c>
-      <c r="Y8" s="337"/>
-      <c r="Z8" s="337"/>
-      <c r="AA8" s="338"/>
-      <c r="AB8" s="339" t="s">
+      <c r="Y8" s="326"/>
+      <c r="Z8" s="326"/>
+      <c r="AA8" s="327"/>
+      <c r="AB8" s="334" t="s">
         <v>199</v>
       </c>
-      <c r="AC8" s="341" t="s">
+      <c r="AC8" s="336" t="s">
         <v>200</v>
       </c>
-      <c r="AD8" s="342"/>
-      <c r="AE8" s="342"/>
-      <c r="AF8" s="342"/>
-      <c r="AG8" s="342"/>
-      <c r="AH8" s="342"/>
+      <c r="AD8" s="337"/>
+      <c r="AE8" s="337"/>
+      <c r="AF8" s="337"/>
+      <c r="AG8" s="337"/>
+      <c r="AH8" s="337"/>
       <c r="AI8" s="328" t="s">
         <v>201</v>
       </c>
@@ -42333,63 +42367,63 @@
       <c r="AL8" s="328"/>
       <c r="AM8" s="328"/>
       <c r="AN8" s="328"/>
-      <c r="AO8" s="324" t="s">
+      <c r="AO8" s="321" t="s">
         <v>202</v>
       </c>
-      <c r="AP8" s="324"/>
-      <c r="AQ8" s="324"/>
-      <c r="AR8" s="324"/>
-      <c r="AS8" s="325" t="s">
+      <c r="AP8" s="321"/>
+      <c r="AQ8" s="321"/>
+      <c r="AR8" s="321"/>
+      <c r="AS8" s="322" t="s">
         <v>203</v>
       </c>
-      <c r="AT8" s="325"/>
-      <c r="AU8" s="325"/>
+      <c r="AT8" s="322"/>
+      <c r="AU8" s="322"/>
       <c r="AV8" s="14"/>
       <c r="AW8" s="14"/>
       <c r="AX8" s="14"/>
       <c r="AY8" s="14"/>
     </row>
     <row r="9" spans="3:54" s="2" customFormat="1" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="330" t="s">
+      <c r="C9" s="323" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="330"/>
-      <c r="E9" s="330"/>
-      <c r="F9" s="330"/>
-      <c r="G9" s="330"/>
-      <c r="H9" s="330"/>
-      <c r="I9" s="330"/>
-      <c r="J9" s="331" t="s">
+      <c r="D9" s="323"/>
+      <c r="E9" s="323"/>
+      <c r="F9" s="323"/>
+      <c r="G9" s="323"/>
+      <c r="H9" s="323"/>
+      <c r="I9" s="323"/>
+      <c r="J9" s="324" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="331"/>
-      <c r="L9" s="331"/>
-      <c r="M9" s="331"/>
-      <c r="N9" s="331"/>
-      <c r="O9" s="331"/>
-      <c r="P9" s="331"/>
-      <c r="Q9" s="331"/>
+      <c r="K9" s="324"/>
+      <c r="L9" s="324"/>
+      <c r="M9" s="324"/>
+      <c r="N9" s="324"/>
+      <c r="O9" s="324"/>
+      <c r="P9" s="324"/>
+      <c r="Q9" s="324"/>
       <c r="R9" s="81"/>
       <c r="S9" s="82"/>
       <c r="T9" s="82"/>
       <c r="U9" s="82"/>
-      <c r="V9" s="336" t="s">
+      <c r="V9" s="325" t="s">
         <v>208</v>
       </c>
-      <c r="W9" s="337"/>
-      <c r="X9" s="337"/>
-      <c r="Y9" s="337"/>
-      <c r="Z9" s="337"/>
-      <c r="AA9" s="338"/>
-      <c r="AB9" s="340"/>
-      <c r="AC9" s="343" t="s">
+      <c r="W9" s="326"/>
+      <c r="X9" s="326"/>
+      <c r="Y9" s="326"/>
+      <c r="Z9" s="326"/>
+      <c r="AA9" s="327"/>
+      <c r="AB9" s="335"/>
+      <c r="AC9" s="346" t="s">
         <v>209</v>
       </c>
-      <c r="AD9" s="343"/>
-      <c r="AE9" s="343"/>
-      <c r="AF9" s="343"/>
-      <c r="AG9" s="343"/>
-      <c r="AH9" s="343"/>
+      <c r="AD9" s="346"/>
+      <c r="AE9" s="346"/>
+      <c r="AF9" s="346"/>
+      <c r="AG9" s="346"/>
+      <c r="AH9" s="346"/>
       <c r="AI9" s="329" t="s">
         <v>201</v>
       </c>
@@ -42398,17 +42432,17 @@
       <c r="AL9" s="329"/>
       <c r="AM9" s="329"/>
       <c r="AN9" s="329"/>
-      <c r="AO9" s="326" t="s">
+      <c r="AO9" s="317" t="s">
         <v>210</v>
       </c>
-      <c r="AP9" s="326"/>
-      <c r="AQ9" s="326"/>
-      <c r="AR9" s="326"/>
-      <c r="AS9" s="327" t="s">
+      <c r="AP9" s="317"/>
+      <c r="AQ9" s="317"/>
+      <c r="AR9" s="317"/>
+      <c r="AS9" s="320" t="s">
         <v>211</v>
       </c>
-      <c r="AT9" s="327"/>
-      <c r="AU9" s="327"/>
+      <c r="AT9" s="320"/>
+      <c r="AU9" s="320"/>
       <c r="AV9" s="83" t="s">
         <v>212</v>
       </c>
@@ -48555,11 +48589,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="O3:X4"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AH8"/>
     <mergeCell ref="AO8:AR8"/>
     <mergeCell ref="AS8:AU8"/>
     <mergeCell ref="C9:I9"/>
@@ -48570,6 +48599,11 @@
     <mergeCell ref="AO9:AR9"/>
     <mergeCell ref="AS9:AU9"/>
     <mergeCell ref="AI8:AN8"/>
+    <mergeCell ref="O3:X4"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AH8"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M67 M69 M70:N70">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="En Proceso">
@@ -48622,41 +48656,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="350" t="s">
+      <c r="A2" s="351" t="s">
         <v>380</v>
       </c>
-      <c r="B2" s="350"/>
-      <c r="C2" s="350"/>
+      <c r="B2" s="351"/>
+      <c r="C2" s="351"/>
       <c r="D2" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="350" t="s">
+      <c r="E2" s="351" t="s">
         <v>382</v>
       </c>
-      <c r="F2" s="350"/>
+      <c r="F2" s="351"/>
       <c r="G2" s="182" t="s">
         <v>199</v>
       </c>
-      <c r="H2" s="349" t="s">
+      <c r="H2" s="350" t="s">
         <v>383</v>
       </c>
-      <c r="I2" s="349"/>
-      <c r="J2" s="349"/>
-      <c r="K2" s="349" t="s">
+      <c r="I2" s="350"/>
+      <c r="J2" s="350"/>
+      <c r="K2" s="350" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="350"/>
-      <c r="M2" s="350"/>
-      <c r="N2" s="349" t="s">
+      <c r="L2" s="351"/>
+      <c r="M2" s="351"/>
+      <c r="N2" s="350" t="s">
         <v>384</v>
       </c>
-      <c r="O2" s="350"/>
-      <c r="P2" s="350"/>
-      <c r="Q2" s="351"/>
-      <c r="R2" s="349" t="s">
+      <c r="O2" s="351"/>
+      <c r="P2" s="351"/>
+      <c r="Q2" s="352"/>
+      <c r="R2" s="350" t="s">
         <v>211</v>
       </c>
-      <c r="S2" s="350"/>
+      <c r="S2" s="351"/>
     </row>
     <row r="3" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A3" s="85" t="s">
@@ -49166,18 +49200,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -49319,25 +49353,25 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62ABF450-D662-42F6-AC20-132C11E15452}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EEA9B3D-0DA4-4009-82C0-0694809F88AF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="fc092c77-77a9-40ad-ae14-39067143678a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EEA9B3D-0DA4-4009-82C0-0694809F88AF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62ABF450-D662-42F6-AC20-132C11E15452}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fc092c77-77a9-40ad-ae14-39067143678a"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
</commit_message>
<xml_diff>
--- a/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
+++ b/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Reforma_Curricular/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{112CFA50-3194-417D-B4BC-6D8321F8E0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{231C229C-C09A-49C4-8378-079081C262DF}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{112CFA50-3194-417D-B4BC-6D8321F8E0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F01FA218-6C13-44A8-A194-A389AD1F2D50}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{5D2AA78B-CF8F-4F04-8CED-873384612ABA}"/>
   </bookViews>
@@ -27,7 +27,7 @@
     <externalReference r:id="rId10"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Borrador!$C$10:$BM$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Borrador!$C$10:$BM$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Borrador (2)'!$C$8:$AY$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Maestro!$C$10:$BZ$10</definedName>
     <definedName name="TABLA_REV">[1]!Tabla2[#All]</definedName>
@@ -33204,7 +33204,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC881F8-DB0A-4697-B988-05828068AF4E}">
-  <sheetPr filterMode="1"/>
   <dimension ref="C3:BM83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
@@ -33645,7 +33644,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="11" spans="3:65" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:65" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C11" s="22" t="s">
         <v>4</v>
       </c>
@@ -33790,7 +33789,7 @@
       </c>
       <c r="BL11" s="12"/>
     </row>
-    <row r="12" spans="3:65" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:65" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C12" s="22" t="s">
         <v>4</v>
       </c>
@@ -33942,7 +33941,7 @@
       </c>
       <c r="BL12" s="12"/>
     </row>
-    <row r="13" spans="3:65" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:65" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C13" s="22" t="s">
         <v>4</v>
       </c>
@@ -34098,7 +34097,7 @@
       </c>
       <c r="BL13" s="12"/>
     </row>
-    <row r="14" spans="3:65" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:65" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C14" s="22" t="s">
         <v>4</v>
       </c>
@@ -34237,7 +34236,7 @@
       </c>
       <c r="BL14" s="12"/>
     </row>
-    <row r="15" spans="3:65" ht="121.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:65" ht="121.8" x14ac:dyDescent="0.3">
       <c r="C15" s="23" t="s">
         <v>10</v>
       </c>
@@ -34379,7 +34378,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="16" spans="3:65" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:65" ht="55.2" x14ac:dyDescent="0.3">
       <c r="C16" s="23" t="s">
         <v>10</v>
       </c>
@@ -34516,7 +34515,7 @@
       </c>
       <c r="BL16" s="12"/>
     </row>
-    <row r="17" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C17" s="23" t="s">
         <v>10</v>
       </c>
@@ -34643,7 +34642,7 @@
       </c>
       <c r="BL17" s="12"/>
     </row>
-    <row r="18" spans="3:64" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:64" ht="55.2" x14ac:dyDescent="0.3">
       <c r="C18" s="23" t="s">
         <v>10</v>
       </c>
@@ -34797,7 +34796,7 @@
       </c>
       <c r="BL18" s="12"/>
     </row>
-    <row r="19" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C19" s="23" t="s">
         <v>10</v>
       </c>
@@ -34936,7 +34935,7 @@
       </c>
       <c r="BL19" s="12"/>
     </row>
-    <row r="20" spans="3:64" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:64" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C20" s="23" t="s">
         <v>10</v>
       </c>
@@ -35075,7 +35074,7 @@
       </c>
       <c r="BL20" s="12"/>
     </row>
-    <row r="21" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C21" s="23" t="s">
         <v>10</v>
       </c>
@@ -35214,7 +35213,7 @@
       </c>
       <c r="BL21" s="12"/>
     </row>
-    <row r="22" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C22" s="23" t="s">
         <v>10</v>
       </c>
@@ -35353,7 +35352,7 @@
       </c>
       <c r="BL22" s="12"/>
     </row>
-    <row r="23" spans="3:64" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:64" ht="55.2" x14ac:dyDescent="0.3">
       <c r="C23" s="23" t="s">
         <v>10</v>
       </c>
@@ -35507,7 +35506,7 @@
       </c>
       <c r="BL23" s="12"/>
     </row>
-    <row r="24" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C24" s="23" t="s">
         <v>10</v>
       </c>
@@ -35636,7 +35635,7 @@
       </c>
       <c r="BL24" s="12"/>
     </row>
-    <row r="25" spans="3:64" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:64" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C25" s="23" t="s">
         <v>10</v>
       </c>
@@ -35775,7 +35774,7 @@
       </c>
       <c r="BL25" s="12"/>
     </row>
-    <row r="26" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C26" s="24" t="s">
         <v>7</v>
       </c>
@@ -35916,7 +35915,7 @@
       </c>
       <c r="BL26" s="12"/>
     </row>
-    <row r="27" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C27" s="24" t="s">
         <v>7</v>
       </c>
@@ -36055,7 +36054,7 @@
       </c>
       <c r="BL27" s="12"/>
     </row>
-    <row r="28" spans="3:64" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:64" ht="55.2" x14ac:dyDescent="0.3">
       <c r="C28" s="24" t="s">
         <v>7</v>
       </c>
@@ -36363,7 +36362,7 @@
       </c>
       <c r="BL29" s="12"/>
     </row>
-    <row r="30" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C30" s="22" t="s">
         <v>4</v>
       </c>
@@ -36490,7 +36489,7 @@
       </c>
       <c r="BL30" s="12"/>
     </row>
-    <row r="31" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C31" s="22" t="s">
         <v>4</v>
       </c>
@@ -36648,7 +36647,7 @@
       </c>
       <c r="BL31" s="12"/>
     </row>
-    <row r="32" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C32" s="22" t="s">
         <v>4</v>
       </c>
@@ -36806,7 +36805,7 @@
       </c>
       <c r="BL32" s="12"/>
     </row>
-    <row r="33" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C33" s="22" t="s">
         <v>4</v>
       </c>
@@ -36945,7 +36944,7 @@
       </c>
       <c r="BL33" s="12"/>
     </row>
-    <row r="34" spans="3:64" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:64" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C34" s="23" t="s">
         <v>10</v>
       </c>
@@ -37072,7 +37071,7 @@
       </c>
       <c r="BL34" s="12"/>
     </row>
-    <row r="35" spans="3:64" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:64" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C35" s="23" t="s">
         <v>10</v>
       </c>
@@ -37501,7 +37500,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C38" s="24" t="s">
         <v>7</v>
       </c>
@@ -37637,7 +37636,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C39" s="24" t="s">
         <v>7</v>
       </c>
@@ -37790,7 +37789,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="3:64" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:64" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C40" s="22" t="s">
         <v>4</v>
       </c>
@@ -37943,7 +37942,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C41" s="22" t="s">
         <v>4</v>
       </c>
@@ -38096,7 +38095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C42" s="23" t="s">
         <v>10</v>
       </c>
@@ -38387,7 +38386,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C44" s="22" t="s">
         <v>4</v>
       </c>
@@ -38538,7 +38537,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C45" s="24" t="s">
         <v>7</v>
       </c>
@@ -38664,7 +38663,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C46" s="24" t="s">
         <v>7</v>
       </c>
@@ -38802,7 +38801,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C47" s="24" t="s">
         <v>7</v>
       </c>
@@ -38955,7 +38954,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="3:64" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:64" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C48" s="24" t="s">
         <v>7</v>
       </c>
@@ -39106,7 +39105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C49" s="22" t="s">
         <v>4</v>
       </c>
@@ -39232,7 +39231,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C50" s="22" t="s">
         <v>4</v>
       </c>
@@ -39523,7 +39522,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C52" s="22" t="s">
         <v>4</v>
       </c>
@@ -39661,7 +39660,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C53" s="22" t="s">
         <v>4</v>
       </c>
@@ -39799,7 +39798,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C54" s="22" t="s">
         <v>4</v>
       </c>
@@ -39943,7 +39942,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C55" s="24" t="s">
         <v>7</v>
       </c>
@@ -40069,7 +40068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
@@ -40211,7 +40210,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C57" s="23" t="s">
         <v>10</v>
       </c>
@@ -40362,7 +40361,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C58" s="23" t="s">
         <v>10</v>
       </c>
@@ -40488,7 +40487,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C59" s="24" t="s">
         <v>7</v>
       </c>
@@ -40614,7 +40613,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C60" s="24" t="s">
         <v>7</v>
       </c>
@@ -40740,7 +40739,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="61" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C61" s="24" t="s">
         <v>7</v>
       </c>
@@ -40878,7 +40877,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C62" s="22" t="s">
         <v>4</v>
       </c>
@@ -41029,7 +41028,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="63" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C63" s="22" t="s">
         <v>4</v>
       </c>
@@ -41155,7 +41154,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C64" s="22" t="s">
         <v>4</v>
       </c>
@@ -41312,7 +41311,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C65" s="22" t="s">
         <v>4</v>
       </c>
@@ -41463,7 +41462,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C66" s="24" t="s">
         <v>7</v>
       </c>
@@ -41589,7 +41588,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="3:63" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="3:63" ht="69.599999999999994" x14ac:dyDescent="0.3">
       <c r="C67" s="22" t="s">
         <v>4</v>
       </c>
@@ -41715,7 +41714,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C68" s="22" t="s">
         <v>4</v>
       </c>
@@ -41841,7 +41840,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
       <c r="C69" s="22" t="s">
         <v>4</v>
       </c>
@@ -42167,19 +42166,7 @@
     <row r="82" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="83" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="C10:BM70" xr:uid="{FBC881F8-DB0A-4697-B988-05828068AF4E}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Híbrido"/>
-        <filter val="Virtual"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="27">
-      <filters>
-        <filter val="NO"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="C10:BM10" xr:uid="{FBC881F8-DB0A-4697-B988-05828068AF4E}"/>
   <mergeCells count="15">
     <mergeCell ref="O3:X4"/>
     <mergeCell ref="J8:Q8"/>

</xml_diff>

<commit_message>
estrellas rojo y amarillo
</commit_message>
<xml_diff>
--- a/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
+++ b/data/raw/CONTROL MAESTRO DE REFORMA CURRICULAR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Reforma_Curricular/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{A5F284E1-7F0C-4711-B144-6978B10ED4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55B297ED-414A-4844-A21A-651E9B65A9EF}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{A5F284E1-7F0C-4711-B144-6978B10ED4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{482BE175-532B-4CF9-9DD3-523CA398D465}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{5D2AA78B-CF8F-4F04-8CED-873384612ABA}"/>
   </bookViews>
@@ -3805,32 +3805,8 @@
     <xf numFmtId="0" fontId="34" fillId="35" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3853,6 +3829,18 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3867,6 +3855,21 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="68" fillId="26" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -3886,15 +3889,6 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3902,6 +3896,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="48" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3915,9 +3918,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -9207,11 +9207,11 @@
         <v>6</v>
       </c>
       <c r="D3" s="283"/>
-      <c r="E3" s="358" t="s">
+      <c r="E3" s="359" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="359"/>
-      <c r="G3" s="360"/>
+      <c r="F3" s="360"/>
+      <c r="G3" s="361"/>
       <c r="H3" s="281" t="s">
         <v>8</v>
       </c>
@@ -12510,21 +12510,21 @@
       <c r="C20" s="121" t="s">
         <v>147</v>
       </c>
-      <c r="D20" s="361" t="s">
+      <c r="D20" s="362" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="361"/>
-      <c r="F20" s="361"/>
-      <c r="G20" s="362" t="s">
+      <c r="E20" s="362"/>
+      <c r="F20" s="362"/>
+      <c r="G20" s="363" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="362"/>
-      <c r="I20" s="362"/>
-      <c r="J20" s="363" t="s">
+      <c r="H20" s="363"/>
+      <c r="I20" s="363"/>
+      <c r="J20" s="364" t="s">
         <v>6</v>
       </c>
-      <c r="K20" s="363"/>
-      <c r="L20" s="363"/>
+      <c r="K20" s="364"/>
+      <c r="L20" s="364"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C21" s="146"/>
@@ -15967,43 +15967,43 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:78" ht="32.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="337" t="s">
+      <c r="O3" s="354" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="337"/>
-      <c r="Q3" s="337"/>
-      <c r="R3" s="337"/>
-      <c r="S3" s="337"/>
-      <c r="T3" s="337"/>
-      <c r="U3" s="337"/>
-      <c r="V3" s="337"/>
-      <c r="W3" s="337"/>
-      <c r="X3" s="337"/>
-      <c r="Y3" s="337"/>
-      <c r="Z3" s="337"/>
-      <c r="AA3" s="337"/>
-      <c r="AB3" s="337"/>
-      <c r="AC3" s="337"/>
+      <c r="P3" s="354"/>
+      <c r="Q3" s="354"/>
+      <c r="R3" s="354"/>
+      <c r="S3" s="354"/>
+      <c r="T3" s="354"/>
+      <c r="U3" s="354"/>
+      <c r="V3" s="354"/>
+      <c r="W3" s="354"/>
+      <c r="X3" s="354"/>
+      <c r="Y3" s="354"/>
+      <c r="Z3" s="354"/>
+      <c r="AA3" s="354"/>
+      <c r="AB3" s="354"/>
+      <c r="AC3" s="354"/>
     </row>
     <row r="4" spans="3:78" x14ac:dyDescent="0.3">
       <c r="J4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="337"/>
-      <c r="P4" s="337"/>
-      <c r="Q4" s="337"/>
-      <c r="R4" s="337"/>
-      <c r="S4" s="337"/>
-      <c r="T4" s="337"/>
-      <c r="U4" s="337"/>
-      <c r="V4" s="337"/>
-      <c r="W4" s="337"/>
-      <c r="X4" s="337"/>
-      <c r="Y4" s="337"/>
-      <c r="Z4" s="337"/>
-      <c r="AA4" s="337"/>
-      <c r="AB4" s="337"/>
-      <c r="AC4" s="337"/>
+      <c r="O4" s="354"/>
+      <c r="P4" s="354"/>
+      <c r="Q4" s="354"/>
+      <c r="R4" s="354"/>
+      <c r="S4" s="354"/>
+      <c r="T4" s="354"/>
+      <c r="U4" s="354"/>
+      <c r="V4" s="354"/>
+      <c r="W4" s="354"/>
+      <c r="X4" s="354"/>
+      <c r="Y4" s="354"/>
+      <c r="Z4" s="354"/>
+      <c r="AA4" s="354"/>
+      <c r="AB4" s="354"/>
+      <c r="AC4" s="354"/>
     </row>
     <row r="5" spans="3:78" x14ac:dyDescent="0.3">
       <c r="J5" s="3" t="s">
@@ -16032,17 +16032,17 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="338" t="s">
+      <c r="J8" s="345" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="338"/>
-      <c r="L8" s="338"/>
-      <c r="M8" s="338"/>
-      <c r="N8" s="338"/>
-      <c r="O8" s="338"/>
-      <c r="P8" s="338"/>
-      <c r="Q8" s="338"/>
-      <c r="R8" s="338"/>
+      <c r="K8" s="345"/>
+      <c r="L8" s="345"/>
+      <c r="M8" s="345"/>
+      <c r="N8" s="345"/>
+      <c r="O8" s="345"/>
+      <c r="P8" s="345"/>
+      <c r="Q8" s="345"/>
+      <c r="R8" s="345"/>
       <c r="S8" s="5" t="s">
         <v>196</v>
       </c>
@@ -16057,168 +16057,168 @@
       <c r="Z8" s="75"/>
       <c r="AA8" s="75"/>
       <c r="AB8" s="75"/>
-      <c r="AC8" s="339" t="s">
+      <c r="AC8" s="346" t="s">
         <v>198</v>
       </c>
-      <c r="AD8" s="340"/>
-      <c r="AE8" s="340"/>
-      <c r="AF8" s="340"/>
-      <c r="AG8" s="340"/>
-      <c r="AH8" s="341"/>
-      <c r="AI8" s="342" t="s">
+      <c r="AD8" s="347"/>
+      <c r="AE8" s="347"/>
+      <c r="AF8" s="347"/>
+      <c r="AG8" s="347"/>
+      <c r="AH8" s="348"/>
+      <c r="AI8" s="355" t="s">
         <v>199</v>
       </c>
       <c r="AJ8" s="170"/>
       <c r="AK8" s="170"/>
-      <c r="AL8" s="344" t="s">
+      <c r="AL8" s="357" t="s">
         <v>200</v>
       </c>
-      <c r="AM8" s="345"/>
-      <c r="AN8" s="345"/>
-      <c r="AO8" s="345"/>
-      <c r="AP8" s="345"/>
-      <c r="AQ8" s="345"/>
-      <c r="AR8" s="353" t="s">
+      <c r="AM8" s="358"/>
+      <c r="AN8" s="358"/>
+      <c r="AO8" s="358"/>
+      <c r="AP8" s="358"/>
+      <c r="AQ8" s="358"/>
+      <c r="AR8" s="349" t="s">
         <v>201</v>
       </c>
-      <c r="AS8" s="353"/>
-      <c r="AT8" s="353"/>
-      <c r="AU8" s="353"/>
-      <c r="AV8" s="353"/>
-      <c r="AW8" s="353"/>
-      <c r="AX8" s="353"/>
-      <c r="AY8" s="353"/>
-      <c r="AZ8" s="353"/>
+      <c r="AS8" s="349"/>
+      <c r="AT8" s="349"/>
+      <c r="AU8" s="349"/>
+      <c r="AV8" s="349"/>
+      <c r="AW8" s="349"/>
+      <c r="AX8" s="349"/>
+      <c r="AY8" s="349"/>
+      <c r="AZ8" s="349"/>
       <c r="BA8" s="174"/>
       <c r="BB8" s="174"/>
       <c r="BC8" s="174"/>
-      <c r="BD8" s="350" t="s">
+      <c r="BD8" s="342" t="s">
         <v>202</v>
       </c>
-      <c r="BE8" s="350"/>
-      <c r="BF8" s="350"/>
-      <c r="BG8" s="350"/>
-      <c r="BH8" s="350"/>
-      <c r="BI8" s="350"/>
-      <c r="BJ8" s="350"/>
-      <c r="BK8" s="350"/>
-      <c r="BL8" s="350"/>
-      <c r="BM8" s="350"/>
-      <c r="BN8" s="350"/>
-      <c r="BO8" s="350"/>
-      <c r="BP8" s="350"/>
-      <c r="BQ8" s="351" t="s">
+      <c r="BE8" s="342"/>
+      <c r="BF8" s="342"/>
+      <c r="BG8" s="342"/>
+      <c r="BH8" s="342"/>
+      <c r="BI8" s="342"/>
+      <c r="BJ8" s="342"/>
+      <c r="BK8" s="342"/>
+      <c r="BL8" s="342"/>
+      <c r="BM8" s="342"/>
+      <c r="BN8" s="342"/>
+      <c r="BO8" s="342"/>
+      <c r="BP8" s="342"/>
+      <c r="BQ8" s="343" t="s">
         <v>203</v>
       </c>
-      <c r="BR8" s="351"/>
-      <c r="BS8" s="351"/>
+      <c r="BR8" s="343"/>
+      <c r="BS8" s="343"/>
       <c r="BT8" s="14"/>
       <c r="BU8" s="14"/>
       <c r="BV8" s="14"/>
       <c r="BW8" s="14"/>
     </row>
     <row r="9" spans="3:78" s="2" customFormat="1" ht="58.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="352" t="s">
+      <c r="C9" s="344" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="352"/>
-      <c r="E9" s="352"/>
-      <c r="F9" s="352"/>
-      <c r="G9" s="352"/>
-      <c r="H9" s="352"/>
-      <c r="I9" s="352"/>
-      <c r="J9" s="338" t="s">
+      <c r="D9" s="344"/>
+      <c r="E9" s="344"/>
+      <c r="F9" s="344"/>
+      <c r="G9" s="344"/>
+      <c r="H9" s="344"/>
+      <c r="I9" s="344"/>
+      <c r="J9" s="345" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="338"/>
-      <c r="L9" s="338"/>
-      <c r="M9" s="338"/>
-      <c r="N9" s="338"/>
-      <c r="O9" s="338"/>
-      <c r="P9" s="338"/>
-      <c r="Q9" s="338"/>
-      <c r="R9" s="338"/>
-      <c r="S9" s="366" t="s">
+      <c r="K9" s="345"/>
+      <c r="L9" s="345"/>
+      <c r="M9" s="345"/>
+      <c r="N9" s="345"/>
+      <c r="O9" s="345"/>
+      <c r="P9" s="345"/>
+      <c r="Q9" s="345"/>
+      <c r="R9" s="345"/>
+      <c r="S9" s="368" t="s">
         <v>205</v>
       </c>
-      <c r="T9" s="367" t="s">
+      <c r="T9" s="365" t="s">
         <v>206</v>
       </c>
-      <c r="U9" s="367" t="s">
+      <c r="U9" s="365" t="s">
         <v>158</v>
       </c>
-      <c r="V9" s="367" t="s">
+      <c r="V9" s="365" t="s">
         <v>207</v>
       </c>
       <c r="W9" s="198"/>
       <c r="X9" s="198"/>
       <c r="Y9" s="198"/>
       <c r="Z9" s="198"/>
-      <c r="AA9" s="339" t="s">
+      <c r="AA9" s="346" t="s">
         <v>208</v>
       </c>
-      <c r="AB9" s="340"/>
-      <c r="AC9" s="340"/>
-      <c r="AD9" s="340"/>
-      <c r="AE9" s="340"/>
-      <c r="AF9" s="340"/>
-      <c r="AG9" s="340"/>
-      <c r="AH9" s="341"/>
-      <c r="AI9" s="343"/>
+      <c r="AB9" s="347"/>
+      <c r="AC9" s="347"/>
+      <c r="AD9" s="347"/>
+      <c r="AE9" s="347"/>
+      <c r="AF9" s="347"/>
+      <c r="AG9" s="347"/>
+      <c r="AH9" s="348"/>
+      <c r="AI9" s="356"/>
       <c r="AJ9" s="172"/>
       <c r="AK9" s="172"/>
-      <c r="AL9" s="369" t="s">
+      <c r="AL9" s="367" t="s">
         <v>209</v>
       </c>
-      <c r="AM9" s="369"/>
-      <c r="AN9" s="369"/>
-      <c r="AO9" s="369"/>
-      <c r="AP9" s="369"/>
-      <c r="AQ9" s="369"/>
-      <c r="AR9" s="354" t="s">
+      <c r="AM9" s="367"/>
+      <c r="AN9" s="367"/>
+      <c r="AO9" s="367"/>
+      <c r="AP9" s="367"/>
+      <c r="AQ9" s="367"/>
+      <c r="AR9" s="350" t="s">
         <v>201</v>
       </c>
-      <c r="AS9" s="354"/>
-      <c r="AT9" s="354"/>
-      <c r="AU9" s="354"/>
-      <c r="AV9" s="354"/>
-      <c r="AW9" s="354"/>
-      <c r="AX9" s="354"/>
-      <c r="AY9" s="354"/>
-      <c r="AZ9" s="354"/>
+      <c r="AS9" s="350"/>
+      <c r="AT9" s="350"/>
+      <c r="AU9" s="350"/>
+      <c r="AV9" s="350"/>
+      <c r="AW9" s="350"/>
+      <c r="AX9" s="350"/>
+      <c r="AY9" s="350"/>
+      <c r="AZ9" s="350"/>
       <c r="BA9" s="175"/>
       <c r="BB9" s="175"/>
       <c r="BC9" s="175"/>
-      <c r="BD9" s="346" t="s">
+      <c r="BD9" s="338" t="s">
         <v>210</v>
       </c>
-      <c r="BE9" s="346"/>
-      <c r="BF9" s="346"/>
-      <c r="BG9" s="346"/>
-      <c r="BH9" s="346"/>
-      <c r="BI9" s="346"/>
-      <c r="BJ9" s="346"/>
-      <c r="BK9" s="346"/>
-      <c r="BL9" s="346"/>
-      <c r="BM9" s="346"/>
-      <c r="BN9" s="346"/>
-      <c r="BO9" s="346"/>
-      <c r="BP9" s="346"/>
-      <c r="BQ9" s="349" t="s">
+      <c r="BE9" s="338"/>
+      <c r="BF9" s="338"/>
+      <c r="BG9" s="338"/>
+      <c r="BH9" s="338"/>
+      <c r="BI9" s="338"/>
+      <c r="BJ9" s="338"/>
+      <c r="BK9" s="338"/>
+      <c r="BL9" s="338"/>
+      <c r="BM9" s="338"/>
+      <c r="BN9" s="338"/>
+      <c r="BO9" s="338"/>
+      <c r="BP9" s="338"/>
+      <c r="BQ9" s="341" t="s">
         <v>211</v>
       </c>
-      <c r="BR9" s="349"/>
-      <c r="BS9" s="349"/>
-      <c r="BT9" s="364" t="s">
+      <c r="BR9" s="341"/>
+      <c r="BS9" s="341"/>
+      <c r="BT9" s="369" t="s">
         <v>212</v>
       </c>
-      <c r="BU9" s="364" t="s">
+      <c r="BU9" s="369" t="s">
         <v>213</v>
       </c>
-      <c r="BV9" s="364" t="s">
+      <c r="BV9" s="369" t="s">
         <v>214</v>
       </c>
-      <c r="BW9" s="365" t="s">
+      <c r="BW9" s="370" t="s">
         <v>215</v>
       </c>
       <c r="BZ9" s="2" t="s">
@@ -16274,10 +16274,10 @@
       <c r="R10" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="S10" s="366"/>
-      <c r="T10" s="368"/>
-      <c r="U10" s="368"/>
-      <c r="V10" s="368"/>
+      <c r="S10" s="368"/>
+      <c r="T10" s="366"/>
+      <c r="U10" s="366"/>
+      <c r="V10" s="366"/>
       <c r="W10" s="173" t="s">
         <v>205</v>
       </c>
@@ -16403,10 +16403,10 @@
       <c r="BS10" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="BT10" s="364"/>
-      <c r="BU10" s="364"/>
-      <c r="BV10" s="364"/>
-      <c r="BW10" s="365"/>
+      <c r="BT10" s="369"/>
+      <c r="BU10" s="369"/>
+      <c r="BV10" s="369"/>
+      <c r="BW10" s="370"/>
     </row>
     <row r="11" spans="3:78" ht="52.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C11" s="22" t="str">
@@ -33446,6 +33446,21 @@
   </sheetData>
   <autoFilter ref="C10:BZ10" xr:uid="{0DE7F4C8-C4D9-4718-9A45-DE15ED66A68A}"/>
   <mergeCells count="23">
+    <mergeCell ref="BU9:BU10"/>
+    <mergeCell ref="BV9:BV10"/>
+    <mergeCell ref="BW9:BW10"/>
+    <mergeCell ref="BD8:BP8"/>
+    <mergeCell ref="BQ8:BS8"/>
+    <mergeCell ref="BD9:BP9"/>
+    <mergeCell ref="BQ9:BS9"/>
+    <mergeCell ref="BT9:BT10"/>
+    <mergeCell ref="AR8:AZ8"/>
+    <mergeCell ref="AR9:AZ9"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="J9:R9"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
     <mergeCell ref="O3:AC4"/>
     <mergeCell ref="J8:R8"/>
     <mergeCell ref="AC8:AH8"/>
@@ -33454,21 +33469,6 @@
     <mergeCell ref="V9:V10"/>
     <mergeCell ref="AA9:AH9"/>
     <mergeCell ref="AL9:AQ9"/>
-    <mergeCell ref="AR8:AZ8"/>
-    <mergeCell ref="AR9:AZ9"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="J9:R9"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="BU9:BU10"/>
-    <mergeCell ref="BV9:BV10"/>
-    <mergeCell ref="BW9:BW10"/>
-    <mergeCell ref="BD8:BP8"/>
-    <mergeCell ref="BQ8:BS8"/>
-    <mergeCell ref="BD9:BP9"/>
-    <mergeCell ref="BQ9:BS9"/>
-    <mergeCell ref="BT9:BT10"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M69 M70:N70">
     <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="En Proceso">
@@ -33557,6 +33557,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC881F8-DB0A-4697-B988-05828068AF4E}">
+  <sheetPr filterMode="1"/>
   <dimension ref="C1:BM83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
@@ -33600,34 +33601,34 @@
       <c r="AS2" s="316"/>
     </row>
     <row r="3" spans="3:65" ht="32.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="337" t="s">
+      <c r="O3" s="354" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="337"/>
-      <c r="Q3" s="337"/>
-      <c r="R3" s="337"/>
-      <c r="S3" s="337"/>
-      <c r="T3" s="337"/>
-      <c r="U3" s="337"/>
-      <c r="V3" s="337"/>
-      <c r="W3" s="337"/>
-      <c r="X3" s="337"/>
+      <c r="P3" s="354"/>
+      <c r="Q3" s="354"/>
+      <c r="R3" s="354"/>
+      <c r="S3" s="354"/>
+      <c r="T3" s="354"/>
+      <c r="U3" s="354"/>
+      <c r="V3" s="354"/>
+      <c r="W3" s="354"/>
+      <c r="X3" s="354"/>
       <c r="AS3" s="316"/>
     </row>
     <row r="4" spans="3:65" ht="14.4" x14ac:dyDescent="0.3">
       <c r="J4" s="318" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="337"/>
-      <c r="P4" s="337"/>
-      <c r="Q4" s="337"/>
-      <c r="R4" s="337"/>
-      <c r="S4" s="337"/>
-      <c r="T4" s="337"/>
-      <c r="U4" s="337"/>
-      <c r="V4" s="337"/>
-      <c r="W4" s="337"/>
-      <c r="X4" s="337"/>
+      <c r="O4" s="354"/>
+      <c r="P4" s="354"/>
+      <c r="Q4" s="354"/>
+      <c r="R4" s="354"/>
+      <c r="S4" s="354"/>
+      <c r="T4" s="354"/>
+      <c r="U4" s="354"/>
+      <c r="V4" s="354"/>
+      <c r="W4" s="354"/>
+      <c r="X4" s="354"/>
       <c r="AS4" s="316"/>
     </row>
     <row r="5" spans="3:65" ht="14.4" x14ac:dyDescent="0.3">
@@ -33660,16 +33661,16 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="338" t="s">
+      <c r="J8" s="345" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="338"/>
-      <c r="L8" s="338"/>
-      <c r="M8" s="338"/>
-      <c r="N8" s="338"/>
-      <c r="O8" s="338"/>
-      <c r="P8" s="338"/>
-      <c r="Q8" s="338"/>
+      <c r="K8" s="345"/>
+      <c r="L8" s="345"/>
+      <c r="M8" s="345"/>
+      <c r="N8" s="345"/>
+      <c r="O8" s="345"/>
+      <c r="P8" s="345"/>
+      <c r="Q8" s="345"/>
       <c r="R8" s="5" t="s">
         <v>196</v>
       </c>
@@ -33680,133 +33681,133 @@
       </c>
       <c r="V8" s="75"/>
       <c r="W8" s="75"/>
-      <c r="X8" s="339" t="s">
+      <c r="X8" s="346" t="s">
         <v>198</v>
       </c>
-      <c r="Y8" s="340"/>
-      <c r="Z8" s="340"/>
-      <c r="AA8" s="340"/>
-      <c r="AB8" s="341"/>
-      <c r="AC8" s="342" t="s">
+      <c r="Y8" s="347"/>
+      <c r="Z8" s="347"/>
+      <c r="AA8" s="347"/>
+      <c r="AB8" s="348"/>
+      <c r="AC8" s="355" t="s">
         <v>199</v>
       </c>
       <c r="AD8" s="170"/>
       <c r="AE8" s="170"/>
-      <c r="AF8" s="344" t="s">
+      <c r="AF8" s="357" t="s">
         <v>200</v>
       </c>
-      <c r="AG8" s="345"/>
-      <c r="AH8" s="345"/>
-      <c r="AI8" s="345"/>
-      <c r="AJ8" s="345"/>
-      <c r="AK8" s="345"/>
-      <c r="AL8" s="353" t="s">
+      <c r="AG8" s="358"/>
+      <c r="AH8" s="358"/>
+      <c r="AI8" s="358"/>
+      <c r="AJ8" s="358"/>
+      <c r="AK8" s="358"/>
+      <c r="AL8" s="349" t="s">
         <v>201</v>
       </c>
-      <c r="AM8" s="353"/>
-      <c r="AN8" s="353"/>
-      <c r="AO8" s="353"/>
-      <c r="AP8" s="353"/>
-      <c r="AQ8" s="353"/>
-      <c r="AR8" s="353"/>
-      <c r="AS8" s="353"/>
-      <c r="AT8" s="350" t="s">
+      <c r="AM8" s="349"/>
+      <c r="AN8" s="349"/>
+      <c r="AO8" s="349"/>
+      <c r="AP8" s="349"/>
+      <c r="AQ8" s="349"/>
+      <c r="AR8" s="349"/>
+      <c r="AS8" s="349"/>
+      <c r="AT8" s="342" t="s">
         <v>202</v>
       </c>
-      <c r="AU8" s="350"/>
-      <c r="AV8" s="350"/>
-      <c r="AW8" s="350"/>
-      <c r="AX8" s="350"/>
-      <c r="AY8" s="350"/>
-      <c r="AZ8" s="350"/>
-      <c r="BA8" s="350"/>
-      <c r="BB8" s="350"/>
-      <c r="BC8" s="351" t="s">
+      <c r="AU8" s="342"/>
+      <c r="AV8" s="342"/>
+      <c r="AW8" s="342"/>
+      <c r="AX8" s="342"/>
+      <c r="AY8" s="342"/>
+      <c r="AZ8" s="342"/>
+      <c r="BA8" s="342"/>
+      <c r="BB8" s="342"/>
+      <c r="BC8" s="343" t="s">
         <v>203</v>
       </c>
-      <c r="BD8" s="351"/>
-      <c r="BE8" s="351"/>
-      <c r="BF8" s="351"/>
-      <c r="BG8" s="351"/>
-      <c r="BH8" s="351"/>
+      <c r="BD8" s="343"/>
+      <c r="BE8" s="343"/>
+      <c r="BF8" s="343"/>
+      <c r="BG8" s="343"/>
+      <c r="BH8" s="343"/>
       <c r="BI8" s="14"/>
       <c r="BJ8" s="14"/>
       <c r="BK8" s="14"/>
       <c r="BL8" s="14"/>
     </row>
     <row r="9" spans="3:65" s="319" customFormat="1" ht="58.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="352" t="s">
+      <c r="C9" s="344" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="352"/>
-      <c r="E9" s="352"/>
-      <c r="F9" s="352"/>
-      <c r="G9" s="352"/>
-      <c r="H9" s="352"/>
-      <c r="I9" s="352"/>
-      <c r="J9" s="338" t="s">
+      <c r="D9" s="344"/>
+      <c r="E9" s="344"/>
+      <c r="F9" s="344"/>
+      <c r="G9" s="344"/>
+      <c r="H9" s="344"/>
+      <c r="I9" s="344"/>
+      <c r="J9" s="345" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="338"/>
-      <c r="L9" s="338"/>
-      <c r="M9" s="338"/>
-      <c r="N9" s="338"/>
-      <c r="O9" s="338"/>
-      <c r="P9" s="338"/>
-      <c r="Q9" s="338"/>
+      <c r="K9" s="345"/>
+      <c r="L9" s="345"/>
+      <c r="M9" s="345"/>
+      <c r="N9" s="345"/>
+      <c r="O9" s="345"/>
+      <c r="P9" s="345"/>
+      <c r="Q9" s="345"/>
       <c r="R9" s="81"/>
       <c r="S9" s="82"/>
       <c r="T9" s="82"/>
       <c r="U9" s="82"/>
-      <c r="V9" s="339" t="s">
+      <c r="V9" s="346" t="s">
         <v>208</v>
       </c>
-      <c r="W9" s="340"/>
-      <c r="X9" s="340"/>
-      <c r="Y9" s="340"/>
-      <c r="Z9" s="340"/>
-      <c r="AA9" s="340"/>
-      <c r="AB9" s="341"/>
-      <c r="AC9" s="343"/>
-      <c r="AD9" s="355" t="s">
+      <c r="W9" s="347"/>
+      <c r="X9" s="347"/>
+      <c r="Y9" s="347"/>
+      <c r="Z9" s="347"/>
+      <c r="AA9" s="347"/>
+      <c r="AB9" s="348"/>
+      <c r="AC9" s="356"/>
+      <c r="AD9" s="351" t="s">
         <v>209</v>
       </c>
-      <c r="AE9" s="356"/>
-      <c r="AF9" s="356"/>
-      <c r="AG9" s="356"/>
-      <c r="AH9" s="356"/>
-      <c r="AI9" s="356"/>
-      <c r="AJ9" s="356"/>
-      <c r="AK9" s="357"/>
-      <c r="AL9" s="354" t="s">
+      <c r="AE9" s="352"/>
+      <c r="AF9" s="352"/>
+      <c r="AG9" s="352"/>
+      <c r="AH9" s="352"/>
+      <c r="AI9" s="352"/>
+      <c r="AJ9" s="352"/>
+      <c r="AK9" s="353"/>
+      <c r="AL9" s="350" t="s">
         <v>201</v>
       </c>
-      <c r="AM9" s="354"/>
-      <c r="AN9" s="354"/>
-      <c r="AO9" s="354"/>
-      <c r="AP9" s="354"/>
-      <c r="AQ9" s="354"/>
-      <c r="AR9" s="354"/>
-      <c r="AS9" s="354"/>
-      <c r="AT9" s="346" t="s">
+      <c r="AM9" s="350"/>
+      <c r="AN9" s="350"/>
+      <c r="AO9" s="350"/>
+      <c r="AP9" s="350"/>
+      <c r="AQ9" s="350"/>
+      <c r="AR9" s="350"/>
+      <c r="AS9" s="350"/>
+      <c r="AT9" s="338" t="s">
         <v>210</v>
       </c>
-      <c r="AU9" s="346"/>
-      <c r="AV9" s="346"/>
-      <c r="AW9" s="346"/>
-      <c r="AX9" s="346"/>
-      <c r="AY9" s="347"/>
-      <c r="AZ9" s="347"/>
-      <c r="BA9" s="347"/>
-      <c r="BB9" s="347"/>
-      <c r="BC9" s="348" t="s">
+      <c r="AU9" s="338"/>
+      <c r="AV9" s="338"/>
+      <c r="AW9" s="338"/>
+      <c r="AX9" s="338"/>
+      <c r="AY9" s="339"/>
+      <c r="AZ9" s="339"/>
+      <c r="BA9" s="339"/>
+      <c r="BB9" s="339"/>
+      <c r="BC9" s="340" t="s">
         <v>211</v>
       </c>
-      <c r="BD9" s="349"/>
-      <c r="BE9" s="349"/>
-      <c r="BF9" s="349"/>
-      <c r="BG9" s="349"/>
-      <c r="BH9" s="349"/>
+      <c r="BD9" s="341"/>
+      <c r="BE9" s="341"/>
+      <c r="BF9" s="341"/>
+      <c r="BG9" s="341"/>
+      <c r="BH9" s="341"/>
       <c r="BI9" s="83" t="s">
         <v>212</v>
       </c>
@@ -34014,7 +34015,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="11" spans="3:65" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:65" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C11" s="22" t="s">
         <v>4</v>
       </c>
@@ -34163,7 +34164,7 @@
       </c>
       <c r="BL11" s="12"/>
     </row>
-    <row r="12" spans="3:65" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:65" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C12" s="22" t="s">
         <v>4</v>
       </c>
@@ -34478,7 +34479,7 @@
       </c>
       <c r="BL13" s="12"/>
     </row>
-    <row r="14" spans="3:65" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:65" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C14" s="22" t="s">
         <v>4</v>
       </c>
@@ -34617,7 +34618,7 @@
       </c>
       <c r="BL14" s="12"/>
     </row>
-    <row r="15" spans="3:65" customFormat="1" ht="121.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:65" customFormat="1" ht="121.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="C15" s="23" t="s">
         <v>10</v>
       </c>
@@ -34761,7 +34762,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="16" spans="3:65" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:65" customFormat="1" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C16" s="23" t="s">
         <v>10</v>
       </c>
@@ -34911,7 +34912,7 @@
       </c>
       <c r="BL16" s="12"/>
     </row>
-    <row r="17" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C17" s="23" t="s">
         <v>10</v>
       </c>
@@ -35065,7 +35066,7 @@
       </c>
       <c r="BL17" s="12"/>
     </row>
-    <row r="18" spans="3:64" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:64" customFormat="1" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C18" s="23" t="s">
         <v>10</v>
       </c>
@@ -35219,7 +35220,7 @@
       </c>
       <c r="BL18" s="12"/>
     </row>
-    <row r="19" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C19" s="23" t="s">
         <v>10</v>
       </c>
@@ -35367,7 +35368,7 @@
       </c>
       <c r="BL19" s="12"/>
     </row>
-    <row r="20" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C20" s="23" t="s">
         <v>10</v>
       </c>
@@ -35515,7 +35516,7 @@
       </c>
       <c r="BL20" s="12"/>
     </row>
-    <row r="21" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C21" s="23" t="s">
         <v>10</v>
       </c>
@@ -35663,7 +35664,7 @@
       </c>
       <c r="BL21" s="12"/>
     </row>
-    <row r="22" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C22" s="23" t="s">
         <v>10</v>
       </c>
@@ -35811,7 +35812,7 @@
       </c>
       <c r="BL22" s="12"/>
     </row>
-    <row r="23" spans="3:64" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:64" customFormat="1" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C23" s="23" t="s">
         <v>10</v>
       </c>
@@ -35904,7 +35905,7 @@
       </c>
       <c r="AI23" s="11"/>
       <c r="AJ23" s="11"/>
-      <c r="AK23" s="374">
+      <c r="AK23" s="337">
         <v>6.25E-2</v>
       </c>
       <c r="AL23" s="12" t="s">
@@ -35965,7 +35966,7 @@
       </c>
       <c r="BL23" s="12"/>
     </row>
-    <row r="24" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C24" s="23" t="s">
         <v>10</v>
       </c>
@@ -36110,7 +36111,7 @@
       </c>
       <c r="BL24" s="12"/>
     </row>
-    <row r="25" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C25" s="23" t="s">
         <v>10</v>
       </c>
@@ -36258,7 +36259,7 @@
       </c>
       <c r="BL25" s="12"/>
     </row>
-    <row r="26" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C26" s="24" t="s">
         <v>7</v>
       </c>
@@ -36399,7 +36400,7 @@
       </c>
       <c r="BL26" s="12"/>
     </row>
-    <row r="27" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C27" s="24" t="s">
         <v>7</v>
       </c>
@@ -36547,7 +36548,7 @@
       </c>
       <c r="BL27" s="12"/>
     </row>
-    <row r="28" spans="3:64" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:64" customFormat="1" ht="55.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C28" s="24" t="s">
         <v>7</v>
       </c>
@@ -36701,7 +36702,7 @@
       </c>
       <c r="BL28" s="12"/>
     </row>
-    <row r="29" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C29" s="23" t="s">
         <v>10</v>
       </c>
@@ -36854,7 +36855,7 @@
       </c>
       <c r="BL29" s="12"/>
     </row>
-    <row r="30" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C30" s="22" t="s">
         <v>4</v>
       </c>
@@ -37009,7 +37010,7 @@
       </c>
       <c r="BL30" s="12"/>
     </row>
-    <row r="31" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C31" s="22" t="s">
         <v>4</v>
       </c>
@@ -37166,7 +37167,7 @@
       </c>
       <c r="BL31" s="12"/>
     </row>
-    <row r="32" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C32" s="22" t="s">
         <v>4</v>
       </c>
@@ -37324,7 +37325,7 @@
       </c>
       <c r="BL32" s="12"/>
     </row>
-    <row r="33" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C33" s="22" t="s">
         <v>4</v>
       </c>
@@ -37472,7 +37473,7 @@
       </c>
       <c r="BL33" s="12"/>
     </row>
-    <row r="34" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C34" s="23" t="s">
         <v>10</v>
       </c>
@@ -37627,7 +37628,7 @@
       </c>
       <c r="BL34" s="12"/>
     </row>
-    <row r="35" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C35" s="23" t="s">
         <v>10</v>
       </c>
@@ -37775,7 +37776,7 @@
       </c>
       <c r="BL35" s="12"/>
     </row>
-    <row r="36" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C36" s="24" t="s">
         <v>7</v>
       </c>
@@ -37933,7 +37934,7 @@
       </c>
       <c r="BL36" s="12"/>
     </row>
-    <row r="37" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C37" s="24" t="s">
         <v>7</v>
       </c>
@@ -38073,7 +38074,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C38" s="24" t="s">
         <v>7</v>
       </c>
@@ -38220,7 +38221,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C39" s="24" t="s">
         <v>7</v>
       </c>
@@ -38373,7 +38374,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="3:64" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:64" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C40" s="22" t="s">
         <v>4</v>
       </c>
@@ -38525,7 +38526,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C41" s="22" t="s">
         <v>4</v>
       </c>
@@ -38684,7 +38685,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C42" s="23" t="s">
         <v>10</v>
       </c>
@@ -38831,7 +38832,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C43" s="23" t="s">
         <v>10</v>
       </c>
@@ -38983,7 +38984,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C44" s="22" t="s">
         <v>4</v>
       </c>
@@ -39140,7 +39141,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C45" s="24" t="s">
         <v>7</v>
       </c>
@@ -39293,7 +39294,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C46" s="24" t="s">
         <v>7</v>
       </c>
@@ -39442,7 +39443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C47" s="24" t="s">
         <v>7</v>
       </c>
@@ -39594,7 +39595,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="3:64" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:64" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C48" s="24" t="s">
         <v>7</v>
       </c>
@@ -39751,7 +39752,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C49" s="22" t="s">
         <v>4</v>
       </c>
@@ -39901,7 +39902,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C50" s="22" t="s">
         <v>4</v>
       </c>
@@ -40050,7 +40051,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="51" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C51" s="24" t="s">
         <v>7</v>
       </c>
@@ -40203,7 +40204,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C52" s="22" t="s">
         <v>4</v>
       </c>
@@ -40352,7 +40353,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C53" s="22" t="s">
         <v>4</v>
       </c>
@@ -40501,7 +40502,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C54" s="22" t="s">
         <v>4</v>
       </c>
@@ -40645,7 +40646,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C55" s="24" t="s">
         <v>7</v>
       </c>
@@ -40798,7 +40799,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
@@ -40946,7 +40947,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C57" s="23" t="s">
         <v>10</v>
       </c>
@@ -41103,7 +41104,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C58" s="23" t="s">
         <v>10</v>
       </c>
@@ -41256,7 +41257,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C59" s="24" t="s">
         <v>7</v>
       </c>
@@ -41409,7 +41410,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C60" s="24" t="s">
         <v>7</v>
       </c>
@@ -41562,7 +41563,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="61" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C61" s="24" t="s">
         <v>7</v>
       </c>
@@ -41711,7 +41712,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C62" s="22" t="s">
         <v>4</v>
       </c>
@@ -41868,7 +41869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="63" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C63" s="22" t="s">
         <v>4</v>
       </c>
@@ -42021,7 +42022,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="3:63" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:63" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C64" s="22" t="s">
         <v>4</v>
       </c>
@@ -42177,7 +42178,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="65" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C65" s="22" t="s">
         <v>4</v>
       </c>
@@ -42334,7 +42335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="66" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C66" s="24" t="s">
         <v>7</v>
       </c>
@@ -42488,7 +42489,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="3:63" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.3">
+    <row r="67" spans="3:63" customFormat="1" ht="69.599999999999994" hidden="1" x14ac:dyDescent="0.3">
       <c r="C67" s="22" t="s">
         <v>4</v>
       </c>
@@ -42643,7 +42644,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="68" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C68" s="22" t="s">
         <v>4</v>
       </c>
@@ -42798,7 +42799,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="69" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C69" s="22" t="s">
         <v>4</v>
       </c>
@@ -42959,7 +42960,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="3:63" customFormat="1" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="70" spans="3:63" customFormat="1" ht="52.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="C70" s="22" t="s">
         <v>4</v>
       </c>
@@ -43136,7 +43137,19 @@
     <row r="82" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="83" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <autoFilter ref="C10:BM70" xr:uid="{FBC881F8-DB0A-4697-B988-05828068AF4E}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Técnica Profesional Judicial"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="15">
+    <mergeCell ref="O3:X4"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="X8:AB8"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AF8:AK8"/>
     <mergeCell ref="AT9:BB9"/>
     <mergeCell ref="BC9:BH9"/>
     <mergeCell ref="AT8:BB8"/>
@@ -43147,11 +43160,6 @@
     <mergeCell ref="AL8:AS8"/>
     <mergeCell ref="AL9:AS9"/>
     <mergeCell ref="AD9:AK9"/>
-    <mergeCell ref="O3:X4"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="X8:AB8"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AF8:AK8"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M67 M69 M70:N70">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="En Proceso">
@@ -43192,10 +43200,10 @@
   </cols>
   <sheetData>
     <row r="10" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D10" s="370" t="s">
+      <c r="D10" s="371" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="370"/>
+      <c r="E10" s="371"/>
     </row>
     <row r="11" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D11" s="329" t="s">
@@ -43388,33 +43396,33 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:54" ht="32.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O3" s="337" t="s">
+      <c r="O3" s="354" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="337"/>
-      <c r="Q3" s="337"/>
-      <c r="R3" s="337"/>
-      <c r="S3" s="337"/>
-      <c r="T3" s="337"/>
-      <c r="U3" s="337"/>
-      <c r="V3" s="337"/>
-      <c r="W3" s="337"/>
-      <c r="X3" s="337"/>
+      <c r="P3" s="354"/>
+      <c r="Q3" s="354"/>
+      <c r="R3" s="354"/>
+      <c r="S3" s="354"/>
+      <c r="T3" s="354"/>
+      <c r="U3" s="354"/>
+      <c r="V3" s="354"/>
+      <c r="W3" s="354"/>
+      <c r="X3" s="354"/>
     </row>
     <row r="4" spans="3:54" x14ac:dyDescent="0.3">
       <c r="J4" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="O4" s="337"/>
-      <c r="P4" s="337"/>
-      <c r="Q4" s="337"/>
-      <c r="R4" s="337"/>
-      <c r="S4" s="337"/>
-      <c r="T4" s="337"/>
-      <c r="U4" s="337"/>
-      <c r="V4" s="337"/>
-      <c r="W4" s="337"/>
-      <c r="X4" s="337"/>
+      <c r="O4" s="354"/>
+      <c r="P4" s="354"/>
+      <c r="Q4" s="354"/>
+      <c r="R4" s="354"/>
+      <c r="S4" s="354"/>
+      <c r="T4" s="354"/>
+      <c r="U4" s="354"/>
+      <c r="V4" s="354"/>
+      <c r="W4" s="354"/>
+      <c r="X4" s="354"/>
     </row>
     <row r="5" spans="3:54" x14ac:dyDescent="0.3">
       <c r="J5" s="3" t="s">
@@ -43443,16 +43451,16 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="77"/>
-      <c r="J8" s="338" t="s">
+      <c r="J8" s="345" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="338"/>
-      <c r="L8" s="338"/>
-      <c r="M8" s="338"/>
-      <c r="N8" s="338"/>
-      <c r="O8" s="338"/>
-      <c r="P8" s="338"/>
-      <c r="Q8" s="338"/>
+      <c r="K8" s="345"/>
+      <c r="L8" s="345"/>
+      <c r="M8" s="345"/>
+      <c r="N8" s="345"/>
+      <c r="O8" s="345"/>
+      <c r="P8" s="345"/>
+      <c r="Q8" s="345"/>
       <c r="R8" s="5" t="s">
         <v>196</v>
       </c>
@@ -43463,107 +43471,107 @@
       </c>
       <c r="V8" s="75"/>
       <c r="W8" s="75"/>
-      <c r="X8" s="339" t="s">
+      <c r="X8" s="346" t="s">
         <v>198</v>
       </c>
-      <c r="Y8" s="340"/>
-      <c r="Z8" s="340"/>
-      <c r="AA8" s="341"/>
-      <c r="AB8" s="342" t="s">
+      <c r="Y8" s="347"/>
+      <c r="Z8" s="347"/>
+      <c r="AA8" s="348"/>
+      <c r="AB8" s="355" t="s">
         <v>199</v>
       </c>
-      <c r="AC8" s="344" t="s">
+      <c r="AC8" s="357" t="s">
         <v>200</v>
       </c>
-      <c r="AD8" s="345"/>
-      <c r="AE8" s="345"/>
-      <c r="AF8" s="345"/>
-      <c r="AG8" s="345"/>
-      <c r="AH8" s="345"/>
-      <c r="AI8" s="353" t="s">
+      <c r="AD8" s="358"/>
+      <c r="AE8" s="358"/>
+      <c r="AF8" s="358"/>
+      <c r="AG8" s="358"/>
+      <c r="AH8" s="358"/>
+      <c r="AI8" s="349" t="s">
         <v>201</v>
       </c>
-      <c r="AJ8" s="353"/>
-      <c r="AK8" s="353"/>
-      <c r="AL8" s="353"/>
-      <c r="AM8" s="353"/>
-      <c r="AN8" s="353"/>
-      <c r="AO8" s="350" t="s">
+      <c r="AJ8" s="349"/>
+      <c r="AK8" s="349"/>
+      <c r="AL8" s="349"/>
+      <c r="AM8" s="349"/>
+      <c r="AN8" s="349"/>
+      <c r="AO8" s="342" t="s">
         <v>202</v>
       </c>
-      <c r="AP8" s="350"/>
-      <c r="AQ8" s="350"/>
-      <c r="AR8" s="350"/>
-      <c r="AS8" s="351" t="s">
+      <c r="AP8" s="342"/>
+      <c r="AQ8" s="342"/>
+      <c r="AR8" s="342"/>
+      <c r="AS8" s="343" t="s">
         <v>203</v>
       </c>
-      <c r="AT8" s="351"/>
-      <c r="AU8" s="351"/>
+      <c r="AT8" s="343"/>
+      <c r="AU8" s="343"/>
       <c r="AV8" s="14"/>
       <c r="AW8" s="14"/>
       <c r="AX8" s="14"/>
       <c r="AY8" s="14"/>
     </row>
     <row r="9" spans="3:54" s="2" customFormat="1" ht="58.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="352" t="s">
+      <c r="C9" s="344" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="352"/>
-      <c r="E9" s="352"/>
-      <c r="F9" s="352"/>
-      <c r="G9" s="352"/>
-      <c r="H9" s="352"/>
-      <c r="I9" s="352"/>
-      <c r="J9" s="338" t="s">
+      <c r="D9" s="344"/>
+      <c r="E9" s="344"/>
+      <c r="F9" s="344"/>
+      <c r="G9" s="344"/>
+      <c r="H9" s="344"/>
+      <c r="I9" s="344"/>
+      <c r="J9" s="345" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="338"/>
-      <c r="L9" s="338"/>
-      <c r="M9" s="338"/>
-      <c r="N9" s="338"/>
-      <c r="O9" s="338"/>
-      <c r="P9" s="338"/>
-      <c r="Q9" s="338"/>
+      <c r="K9" s="345"/>
+      <c r="L9" s="345"/>
+      <c r="M9" s="345"/>
+      <c r="N9" s="345"/>
+      <c r="O9" s="345"/>
+      <c r="P9" s="345"/>
+      <c r="Q9" s="345"/>
       <c r="R9" s="81"/>
       <c r="S9" s="82"/>
       <c r="T9" s="82"/>
       <c r="U9" s="82"/>
-      <c r="V9" s="339" t="s">
+      <c r="V9" s="346" t="s">
         <v>208</v>
       </c>
-      <c r="W9" s="340"/>
-      <c r="X9" s="340"/>
-      <c r="Y9" s="340"/>
-      <c r="Z9" s="340"/>
-      <c r="AA9" s="341"/>
-      <c r="AB9" s="343"/>
-      <c r="AC9" s="369" t="s">
+      <c r="W9" s="347"/>
+      <c r="X9" s="347"/>
+      <c r="Y9" s="347"/>
+      <c r="Z9" s="347"/>
+      <c r="AA9" s="348"/>
+      <c r="AB9" s="356"/>
+      <c r="AC9" s="367" t="s">
         <v>209</v>
       </c>
-      <c r="AD9" s="369"/>
-      <c r="AE9" s="369"/>
-      <c r="AF9" s="369"/>
-      <c r="AG9" s="369"/>
-      <c r="AH9" s="369"/>
-      <c r="AI9" s="354" t="s">
+      <c r="AD9" s="367"/>
+      <c r="AE9" s="367"/>
+      <c r="AF9" s="367"/>
+      <c r="AG9" s="367"/>
+      <c r="AH9" s="367"/>
+      <c r="AI9" s="350" t="s">
         <v>201</v>
       </c>
-      <c r="AJ9" s="354"/>
-      <c r="AK9" s="354"/>
-      <c r="AL9" s="354"/>
-      <c r="AM9" s="354"/>
-      <c r="AN9" s="354"/>
-      <c r="AO9" s="346" t="s">
+      <c r="AJ9" s="350"/>
+      <c r="AK9" s="350"/>
+      <c r="AL9" s="350"/>
+      <c r="AM9" s="350"/>
+      <c r="AN9" s="350"/>
+      <c r="AO9" s="338" t="s">
         <v>210</v>
       </c>
-      <c r="AP9" s="346"/>
-      <c r="AQ9" s="346"/>
-      <c r="AR9" s="346"/>
-      <c r="AS9" s="349" t="s">
+      <c r="AP9" s="338"/>
+      <c r="AQ9" s="338"/>
+      <c r="AR9" s="338"/>
+      <c r="AS9" s="341" t="s">
         <v>211</v>
       </c>
-      <c r="AT9" s="349"/>
-      <c r="AU9" s="349"/>
+      <c r="AT9" s="341"/>
+      <c r="AU9" s="341"/>
       <c r="AV9" s="83" t="s">
         <v>212</v>
       </c>
@@ -49710,11 +49718,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="O3:X4"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AH8"/>
     <mergeCell ref="AO8:AR8"/>
     <mergeCell ref="AS8:AU8"/>
     <mergeCell ref="C9:I9"/>
@@ -49725,6 +49728,11 @@
     <mergeCell ref="AO9:AR9"/>
     <mergeCell ref="AS9:AU9"/>
     <mergeCell ref="AI8:AN8"/>
+    <mergeCell ref="O3:X4"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AH8"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M67 M69 M70:N70">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="En Proceso">
@@ -49777,41 +49785,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="372" t="s">
+      <c r="A2" s="373" t="s">
         <v>391</v>
       </c>
-      <c r="B2" s="372"/>
-      <c r="C2" s="372"/>
+      <c r="B2" s="373"/>
+      <c r="C2" s="373"/>
       <c r="D2" t="s">
         <v>392</v>
       </c>
-      <c r="E2" s="372" t="s">
+      <c r="E2" s="373" t="s">
         <v>393</v>
       </c>
-      <c r="F2" s="372"/>
+      <c r="F2" s="373"/>
       <c r="G2" s="181" t="s">
         <v>199</v>
       </c>
-      <c r="H2" s="371" t="s">
+      <c r="H2" s="372" t="s">
         <v>394</v>
       </c>
-      <c r="I2" s="371"/>
-      <c r="J2" s="371"/>
-      <c r="K2" s="371" t="s">
+      <c r="I2" s="372"/>
+      <c r="J2" s="372"/>
+      <c r="K2" s="372" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="372"/>
-      <c r="M2" s="372"/>
-      <c r="N2" s="371" t="s">
+      <c r="L2" s="373"/>
+      <c r="M2" s="373"/>
+      <c r="N2" s="372" t="s">
         <v>395</v>
       </c>
-      <c r="O2" s="372"/>
-      <c r="P2" s="372"/>
-      <c r="Q2" s="373"/>
-      <c r="R2" s="371" t="s">
+      <c r="O2" s="373"/>
+      <c r="P2" s="373"/>
+      <c r="Q2" s="374"/>
+      <c r="R2" s="372" t="s">
         <v>211</v>
       </c>
-      <c r="S2" s="372"/>
+      <c r="S2" s="373"/>
     </row>
     <row r="3" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A3" s="85" t="s">
@@ -50071,6 +50079,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101009D53C3A3428B1B4A9D164F0D85BEEA57" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="1b756714394f243dc1e59234ebaea7ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fc092c77-77a9-40ad-ae14-39067143678a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47b6ece98d39c8f8132b14d131b38829" ns2:_="">
     <xsd:import namespace="fc092c77-77a9-40ad-ae14-39067143678a"/>
@@ -50208,15 +50225,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EEA9B3D-0DA4-4009-82C0-0694809F88AF}">
   <ds:schemaRefs>
@@ -50227,6 +50235,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62ABF450-D662-42F6-AC20-132C11E15452}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F88112FF-E6D9-4EFB-A2F0-A6CBF29F2F7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -50242,12 +50258,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62ABF450-D662-42F6-AC20-132C11E15452}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>